<commit_message>
feat: update experiment files and remove obsolete result files for cleaner project structure
</commit_message>
<xml_diff>
--- a/tutorial/ecoli/experiments/Δpgi_ecoli.xlsx
+++ b/tutorial/ecoli/experiments/Δpgi_ecoli.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="libxl" lastEdited="7" lowestEdited="6" rupBuild="4.6.0"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="6150" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="6642" uniqueCount="63">
   <si>
     <t>mu</t>
   </si>
@@ -2160,7 +2160,7 @@
         <v>0.60775783940547401</v>
       </c>
       <c r="AI2" s="0">
-        <v>0.6682907764460656</v>
+        <v>0.66829077644606561</v>
       </c>
       <c r="AJ2" s="0">
         <v>0.70667544933498216</v>
@@ -2207,7 +2207,7 @@
         <v>0.18802039431755105</v>
       </c>
       <c r="N3" s="0">
-        <v>0.20918612729118793</v>
+        <v>0.20918612729118794</v>
       </c>
       <c r="O3" s="0">
         <v>0.14069706459361639</v>
@@ -2216,7 +2216,7 @@
         <v>0.30669546436285094</v>
       </c>
       <c r="Q3" s="0">
-        <v>0.22437221364453624</v>
+        <v>0.22437221364453625</v>
       </c>
       <c r="R3" s="0">
         <v>0.21702861965547904</v>
@@ -2433,7 +2433,7 @@
         <v>0.004916444189293892</v>
       </c>
       <c r="P5" s="0">
-        <v>0.02159827213822894</v>
+        <v>0.021598272138228941</v>
       </c>
       <c r="Q5" s="0">
         <v>0.023928401943681364</v>
@@ -2466,7 +2466,7 @@
         <v>0.028990967908624085</v>
       </c>
       <c r="AA5" s="0">
-        <v>0.024037119494543051</v>
+        <v>0.024037119494543052</v>
       </c>
       <c r="AB5" s="0">
         <v>0.01505468079121829</v>
@@ -2864,7 +2864,7 @@
         <v>0.0002521148141591971</v>
       </c>
       <c r="M9" s="0">
-        <v>0.00052424909027363748</v>
+        <v>0.00052424909027363749</v>
       </c>
       <c r="N9" s="0">
         <v>0.00016922282192415256</v>
@@ -2962,7 +2962,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="0">
-        <v>0.00015393386545039909</v>
+        <v>0.0001539338654503991</v>
       </c>
       <c r="J10" s="0">
         <v>5.1450213518386101e-05</v>
@@ -3498,36 +3498,36 @@
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="true"/>
     <col min="2" max="2" width="16.42578125" customWidth="true"/>
-    <col min="3" max="3" width="16.42578125" customWidth="true"/>
-    <col min="4" max="4" width="16.28515625" customWidth="true"/>
+    <col min="3" max="3" width="15.7109375" customWidth="true"/>
+    <col min="4" max="4" width="14.7109375" customWidth="true"/>
     <col min="5" max="5" width="16.28515625" customWidth="true"/>
     <col min="6" max="6" width="16.42578125" customWidth="true"/>
-    <col min="7" max="7" width="16.28515625" customWidth="true"/>
-    <col min="8" max="8" width="16.28515625" customWidth="true"/>
+    <col min="7" max="7" width="14.7109375" customWidth="true"/>
+    <col min="8" max="8" width="16.42578125" customWidth="true"/>
     <col min="9" max="9" width="16.42578125" customWidth="true"/>
-    <col min="10" max="10" width="16.28515625" customWidth="true"/>
+    <col min="10" max="10" width="15.7109375" customWidth="true"/>
     <col min="11" max="11" width="16.42578125" customWidth="true"/>
-    <col min="12" max="12" width="16.28515625" customWidth="true"/>
+    <col min="12" max="12" width="15.7109375" customWidth="true"/>
     <col min="13" max="13" width="16.28515625" customWidth="true"/>
     <col min="14" max="14" width="16.28515625" customWidth="true"/>
     <col min="15" max="15" width="16.42578125" customWidth="true"/>
-    <col min="16" max="16" width="15.5703125" customWidth="true"/>
+    <col min="16" max="16" width="16.28515625" customWidth="true"/>
     <col min="17" max="17" width="16.28515625" customWidth="true"/>
-    <col min="18" max="18" width="16.42578125" customWidth="true"/>
-    <col min="19" max="19" width="16.28515625" customWidth="true"/>
-    <col min="20" max="20" width="16.42578125" customWidth="true"/>
+    <col min="18" max="18" width="15.7109375" customWidth="true"/>
+    <col min="19" max="19" width="15.42578125" customWidth="true"/>
+    <col min="20" max="20" width="14.7109375" customWidth="true"/>
     <col min="21" max="21" width="16.42578125" customWidth="true"/>
     <col min="22" max="22" width="16.42578125" customWidth="true"/>
     <col min="23" max="23" width="15.7109375" customWidth="true"/>
     <col min="24" max="24" width="16.42578125" customWidth="true"/>
-    <col min="25" max="25" width="16.42578125" customWidth="true"/>
+    <col min="25" max="25" width="16.28515625" customWidth="true"/>
     <col min="26" max="26" width="16.28515625" customWidth="true"/>
-    <col min="27" max="27" width="16.28515625" customWidth="true"/>
-    <col min="28" max="28" width="16.28515625" customWidth="true"/>
+    <col min="27" max="27" width="14.7109375" customWidth="true"/>
+    <col min="28" max="28" width="13.7109375" customWidth="true"/>
     <col min="29" max="29" width="16.42578125" customWidth="true"/>
-    <col min="30" max="30" width="16.28515625" customWidth="true"/>
-    <col min="31" max="31" width="16.28515625" customWidth="true"/>
-    <col min="32" max="32" width="16.28515625" customWidth="true"/>
+    <col min="30" max="30" width="15.5703125" customWidth="true"/>
+    <col min="31" max="31" width="15.7109375" customWidth="true"/>
+    <col min="32" max="32" width="15.42578125" customWidth="true"/>
     <col min="33" max="33" width="16.42578125" customWidth="true"/>
     <col min="34" max="34" width="16.42578125" customWidth="true"/>
     <col min="35" max="35" width="16.42578125" customWidth="true"/>
@@ -3649,109 +3649,109 @@
         <v>36</v>
       </c>
       <c r="B2" s="0">
-        <v>0.89404080296762911</v>
+        <v>0.89394703562676636</v>
       </c>
       <c r="C2" s="0">
-        <v>0.99550362427367445</v>
+        <v>0.99514840557432582</v>
       </c>
       <c r="D2" s="0">
-        <v>0.94401786586842185</v>
+        <v>0.94746484268514786</v>
       </c>
       <c r="E2" s="0">
-        <v>0.89387823715521442</v>
+        <v>0.89388697768454184</v>
       </c>
       <c r="F2" s="0">
-        <v>0.99058047310702224</v>
+        <v>0.99057345142567721</v>
       </c>
       <c r="G2" s="0">
-        <v>0.97868581388725973</v>
+        <v>0.97920481428562911</v>
       </c>
       <c r="H2" s="0">
-        <v>0.90334018072714461</v>
+        <v>0.90330541160924072</v>
       </c>
       <c r="I2" s="0">
-        <v>0.99473931457139542</v>
+        <v>0.99498861624680579</v>
       </c>
       <c r="J2" s="0">
-        <v>0.97405780022027477</v>
+        <v>0.97434251081769352</v>
       </c>
       <c r="K2" s="0">
-        <v>0.93188711195237584</v>
+        <v>0.93187936249569137</v>
       </c>
       <c r="L2" s="0">
-        <v>0.92402665556681429</v>
+        <v>0.92436077059679789</v>
       </c>
       <c r="M2" s="0">
-        <v>0.83246690068568308</v>
+        <v>0.83246689355386039</v>
       </c>
       <c r="N2" s="0">
-        <v>0.94153940039465345</v>
+        <v>0.94153938133758508</v>
       </c>
       <c r="O2" s="0">
-        <v>0.98046475824108614</v>
+        <v>0.98046472362608161</v>
       </c>
       <c r="P2" s="0">
-        <v>0.70897761940434434</v>
+        <v>0.70897799349932367</v>
       </c>
       <c r="Q2" s="0">
-        <v>0.998442169919042</v>
+        <v>0.99847034997159656</v>
       </c>
       <c r="R2" s="0">
-        <v>1.0033977604639746</v>
+        <v>1.0032712342662635</v>
       </c>
       <c r="S2" s="0">
-        <v>1.004115749592162</v>
+        <v>1.0044532298401239</v>
       </c>
       <c r="T2" s="0">
-        <v>0.99230163893617074</v>
+        <v>0.99333457561696192</v>
       </c>
       <c r="U2" s="0">
-        <v>0.98993887412151227</v>
+        <v>0.9900711597210049</v>
       </c>
       <c r="V2" s="0">
-        <v>0.99134811373220477</v>
+        <v>0.99365443162119926</v>
       </c>
       <c r="W2" s="0">
-        <v>0.95310707532105432</v>
+        <v>0.99060966912080828</v>
       </c>
       <c r="X2" s="0">
-        <v>0.99040629062860452</v>
+        <v>0.99127250996737959</v>
       </c>
       <c r="Y2" s="0">
-        <v>0.90160625277000805</v>
+        <v>0.90163039287843505</v>
       </c>
       <c r="Z2" s="0">
-        <v>0.93381527312226253</v>
+        <v>0.93384626370114077</v>
       </c>
       <c r="AA2" s="0">
-        <v>0.91873539412130034</v>
+        <v>0.91995500977575284</v>
       </c>
       <c r="AB2" s="0">
-        <v>0.96520033463672805</v>
+        <v>0.96562133962282559</v>
       </c>
       <c r="AC2" s="0">
-        <v>0.92674073641492183</v>
+        <v>0.92674259928014391</v>
       </c>
       <c r="AD2" s="0">
-        <v>1.0015295561303097</v>
+        <v>1.0016317093111582</v>
       </c>
       <c r="AE2" s="0">
-        <v>0.99404477353971354</v>
+        <v>0.99415901258958683</v>
       </c>
       <c r="AF2" s="0">
-        <v>0.89635811818313438</v>
+        <v>0.90956994892389786</v>
       </c>
       <c r="AG2" s="0">
-        <v>0.99255131227799842</v>
+        <v>0.99258699741400613</v>
       </c>
       <c r="AH2" s="0">
-        <v>0.99661233723740239</v>
+        <v>0.99652796909344343</v>
       </c>
       <c r="AI2" s="0">
-        <v>0.98583886928446074</v>
+        <v>0.98581690823711166</v>
       </c>
       <c r="AJ2" s="0">
-        <v>0.97878076022364635</v>
+        <v>0.97878079788661931</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
@@ -3759,109 +3759,109 @@
         <v>37</v>
       </c>
       <c r="B3" s="0">
-        <v>0.10655273893971534</v>
+        <v>0.10540156891673025</v>
       </c>
       <c r="C3" s="0">
-        <v>0.0040738379221342625</v>
+        <v>0.0040288097707927633</v>
       </c>
       <c r="D3" s="0">
-        <v>0.009505421949826412</v>
+        <v>0.0094380505562253279</v>
       </c>
       <c r="E3" s="0">
-        <v>0.10868519024662363</v>
+        <v>0.1075233100862354</v>
       </c>
       <c r="F3" s="0">
-        <v>0.0085083703097420457</v>
+        <v>0.0084172710815895533</v>
       </c>
       <c r="G3" s="0">
-        <v>0.0044308376298045921</v>
+        <v>0.0043857522136883783</v>
       </c>
       <c r="H3" s="0">
-        <v>0.0980587286666708</v>
+        <v>0.097005766422130518</v>
       </c>
       <c r="I3" s="0">
-        <v>0.0049079251002786357</v>
+        <v>0.0048566271651645414</v>
       </c>
       <c r="J3" s="0">
-        <v>0.0091388377088323022</v>
+        <v>0.0090436947845803084</v>
       </c>
       <c r="K3" s="0">
-        <v>0.072041861899509785</v>
+        <v>0.071270421296345685</v>
       </c>
       <c r="L3" s="0">
-        <v>0.069435375992346227</v>
+        <v>0.068717255680316641</v>
       </c>
       <c r="M3" s="0">
-        <v>0.048680863124526214</v>
+        <v>0.048159977476502691</v>
       </c>
       <c r="N3" s="0">
-        <v>0.057096615346514223</v>
+        <v>0.056485680419017671</v>
       </c>
       <c r="O3" s="0">
-        <v>0.0083804489083624291</v>
+        <v>0.0082907778123396322</v>
       </c>
       <c r="P3" s="0">
-        <v>0.2388720144785518</v>
+        <v>0.23631620861679239</v>
       </c>
       <c r="Q3" s="0">
-        <v>0.002770225474618822</v>
+        <v>0.0027406614123418392</v>
       </c>
       <c r="R3" s="0">
-        <v>-0.0035731919045169343</v>
+        <v>-0.0035345130008016699</v>
       </c>
       <c r="S3" s="0">
-        <v>-0.0015662058993536963</v>
+        <v>-0.0015499682608192007</v>
       </c>
       <c r="T3" s="0">
-        <v>0.0026409176004600098</v>
+        <v>0.0026153794310981673</v>
       </c>
       <c r="U3" s="0">
-        <v>0.010626702596346018</v>
+        <v>0.010514401731057468</v>
       </c>
       <c r="V3" s="0">
-        <v>0.0063806819436035486</v>
+        <v>0.0063270941248778616</v>
       </c>
       <c r="W3" s="0">
-        <v>0.0045170787762603692</v>
+        <v>0.0046445810172954412</v>
       </c>
       <c r="X3" s="0">
-        <v>0.0090970296122694187</v>
+        <v>0.0090075626163539091</v>
       </c>
       <c r="Y3" s="0">
-        <v>0.097797084860847913</v>
+        <v>0.096753246508837251</v>
       </c>
       <c r="Z3" s="0">
-        <v>0.06823769401261548</v>
+        <v>0.067509791063481567</v>
       </c>
       <c r="AA3" s="0">
-        <v>0.069327781276378592</v>
+        <v>0.068677021480574266</v>
       </c>
       <c r="AB3" s="0">
-        <v>0.033053742120738978</v>
+        <v>0.03271433032757444</v>
       </c>
       <c r="AC3" s="0">
-        <v>0.074086893883940047</v>
+        <v>0.073294311449853072</v>
       </c>
       <c r="AD3" s="0">
-        <v>-0.0017927299364722557</v>
+        <v>-0.0017737286230016436</v>
       </c>
       <c r="AE3" s="0">
-        <v>0.00392785495245209</v>
+        <v>0.0038862734770754026</v>
       </c>
       <c r="AF3" s="0">
-        <v>0.094267130657389037</v>
+        <v>0.094633051477856597</v>
       </c>
       <c r="AG3" s="0">
-        <v>0.0078252179894272317</v>
+        <v>0.0077417664861857737</v>
       </c>
       <c r="AH3" s="0">
-        <v>0.0018794428105261543</v>
+        <v>0.0018591753707746144</v>
       </c>
       <c r="AI3" s="0">
-        <v>-0.00022172076991240571</v>
+        <v>-0.00021934347135900379</v>
       </c>
       <c r="AJ3" s="0">
-        <v>0.011151227210340129</v>
+        <v>0.011031909503691595</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
@@ -3869,109 +3869,109 @@
         <v>38</v>
       </c>
       <c r="B4" s="0">
-        <v>-0.00027428442084424679</v>
+        <v>0.0008593788050808819</v>
       </c>
       <c r="C4" s="0">
-        <v>0.00079691749142727958</v>
+        <v>0.00082278465488138145</v>
       </c>
       <c r="D4" s="0">
-        <v>0.043771391602916522</v>
+        <v>0.043097106758626734</v>
       </c>
       <c r="E4" s="0">
-        <v>-0.0027000390086994418</v>
+        <v>-0.0014920937230353155</v>
       </c>
       <c r="F4" s="0">
-        <v>0.0018569433279909196</v>
+        <v>0.0019074692601123997</v>
       </c>
       <c r="G4" s="0">
-        <v>0.0043964765706695939</v>
+        <v>0.0043521047132952986</v>
       </c>
       <c r="H4" s="0">
-        <v>-0.0013785344710791046</v>
+        <v>-0.00031117803137135409</v>
       </c>
       <c r="I4" s="0">
-        <v>0.00039908019369331882</v>
+        <v>0.00044264936750459114</v>
       </c>
       <c r="J4" s="0">
-        <v>0.015561466824230328</v>
+        <v>0.015331452296253512</v>
       </c>
       <c r="K4" s="0">
-        <v>-0.0038068056968323383</v>
+        <v>-0.0029631514051470377</v>
       </c>
       <c r="L4" s="0">
-        <v>0.0046848090158769871</v>
+        <v>0.0053220230066635963</v>
       </c>
       <c r="M4" s="0">
-        <v>-0.0062447847493337771</v>
+        <v>-0.0055965495097445002</v>
       </c>
       <c r="N4" s="0">
-        <v>0.00071796835444145799</v>
+        <v>0.0013070827981142229</v>
       </c>
       <c r="O4" s="0">
-        <v>0.0032145605524505419</v>
+        <v>0.0032348482031843949</v>
       </c>
       <c r="P4" s="0">
-        <v>-0.045234060198447369</v>
+        <v>-0.041742670085451114</v>
       </c>
       <c r="Q4" s="0">
-        <v>-0.0012231643377970764</v>
+        <v>-0.0011678373717253971</v>
       </c>
       <c r="R4" s="0">
-        <v>0.00030768523332857373</v>
+        <v>0.00026327873453824705</v>
       </c>
       <c r="S4" s="0">
-        <v>-0.0029484666580938748</v>
+        <v>-0.002903261579304697</v>
       </c>
       <c r="T4" s="0">
-        <v>0.0041052605451564559</v>
+        <v>0.004050044951939928</v>
       </c>
       <c r="U4" s="0">
-        <v>-0.00084235024654027242</v>
+        <v>-0.00071202646077514551</v>
       </c>
       <c r="V4" s="0">
-        <v>-0.00031232550575718457</v>
+        <v>-0.00023868873314848664</v>
       </c>
       <c r="W4" s="0">
-        <v>0.0032937984941461265</v>
+        <v>0.0034002301271040163</v>
       </c>
       <c r="X4" s="0">
-        <v>-0.00038430466213691553</v>
+        <v>-0.00028007258373341905</v>
       </c>
       <c r="Y4" s="0">
-        <v>0.00097790045140512018</v>
+        <v>0.0019923707047487679</v>
       </c>
       <c r="Z4" s="0">
-        <v>-0.0020450522269380936</v>
+        <v>-0.0012792339075608497</v>
       </c>
       <c r="AA4" s="0">
-        <v>0.002154722133328053</v>
+        <v>0.0028465013995376161</v>
       </c>
       <c r="AB4" s="0">
-        <v>0.0013422849130821752</v>
+        <v>0.0016643300495999091</v>
       </c>
       <c r="AC4" s="0">
-        <v>-0.00055748835368217553</v>
+        <v>0.00023862610598987107</v>
       </c>
       <c r="AD4" s="0">
-        <v>4.7664880140986252e-05</v>
+        <v>2.7676170791495158e-05</v>
       </c>
       <c r="AE4" s="0">
-        <v>0.0016614400856144651</v>
+        <v>0.0016678454864591454</v>
       </c>
       <c r="AF4" s="0">
-        <v>-0.0052515989244892548</v>
+        <v>-0.0042030004017544692</v>
       </c>
       <c r="AG4" s="0">
-        <v>-0.0011750250782625938</v>
+        <v>-0.0010672185151916114</v>
       </c>
       <c r="AH4" s="0">
-        <v>-0.0012300094013063341</v>
+        <v>-0.0011838329374547689</v>
       </c>
       <c r="AI4" s="0">
-        <v>0.012058816850129675</v>
+        <v>0.011799528897896837</v>
       </c>
       <c r="AJ4" s="0">
-        <v>0.00058659293197979091</v>
+        <v>0.00069214845604104386</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
@@ -3979,109 +3979,109 @@
         <v>39</v>
       </c>
       <c r="B5" s="0">
-        <v>-0.00022135897231911254</v>
+        <v>-0.00020798334857744576</v>
       </c>
       <c r="C5" s="0">
-        <v>-0.00031406223412518933</v>
+        <v>0</v>
       </c>
       <c r="D5" s="0">
-        <v>0.0010933246548526718</v>
+        <v>0</v>
       </c>
       <c r="E5" s="0">
-        <v>3.7467698143955209e-05</v>
+        <v>-7.9629865484182324e-06</v>
       </c>
       <c r="F5" s="0">
-        <v>-0.00091859800123616619</v>
+        <v>-0.00084956293748116062</v>
       </c>
       <c r="G5" s="0">
-        <v>0.011291962650674102</v>
+        <v>0.01103178617824256</v>
       </c>
       <c r="H5" s="0">
-        <v>2.3100606090794953e-05</v>
+        <v>0</v>
       </c>
       <c r="I5" s="0">
-        <v>-0.00029358495185070866</v>
+        <v>-0.00027541593325629434</v>
       </c>
       <c r="J5" s="0">
-        <v>0.00027019701253181794</v>
+        <v>0.00058875029717742478</v>
       </c>
       <c r="K5" s="0">
-        <v>-0.00010059746734066325</v>
+        <v>-0.00016897309823045935</v>
       </c>
       <c r="L5" s="0">
-        <v>0.00076556089510165944</v>
+        <v>0.00084754027845014991</v>
       </c>
       <c r="M5" s="0">
-        <v>0.10881504428535833</v>
+        <v>0.10523404186599762</v>
       </c>
       <c r="N5" s="0">
-        <v>-6.5817404459698559e-05</v>
+        <v>-4.2222663832970632e-05</v>
       </c>
       <c r="O5" s="0">
-        <v>0.00079774159219915379</v>
+        <v>0.00084068362325329582</v>
       </c>
       <c r="P5" s="0">
-        <v>0.0050410789410492603</v>
+        <v>0.0039606391838060764</v>
       </c>
       <c r="Q5" s="0">
-        <v>-1.8454069649232189e-05</v>
+        <v>-4.3174012212862981e-05</v>
       </c>
       <c r="R5" s="0">
-        <v>-1.6875046374935369e-05</v>
+        <v>0</v>
       </c>
       <c r="S5" s="0">
-        <v>0.00027341521774166367</v>
+        <v>0</v>
       </c>
       <c r="T5" s="0">
-        <v>0.00052167955629449435</v>
+        <v>0</v>
       </c>
       <c r="U5" s="0">
-        <v>4.0971030860580887e-05</v>
+        <v>2.3234023873047627e-05</v>
       </c>
       <c r="V5" s="0">
-        <v>-2.4187829195669044e-05</v>
+        <v>-2.9306490553921093e-05</v>
       </c>
       <c r="W5" s="0">
-        <v>0.00067485948010435795</v>
+        <v>0.00075137150772460002</v>
       </c>
       <c r="X5" s="0">
-        <v>9.3966705985790445e-05</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="0">
-        <v>-0.00037321461382927394</v>
+        <v>-0.00032981237696778914</v>
       </c>
       <c r="Z5" s="0">
-        <v>-4.3082886840458259e-05</v>
+        <v>-7.6820857061364695e-05</v>
       </c>
       <c r="AA5" s="0">
-        <v>0.0087345787941913722</v>
+        <v>0.0085214673441352546</v>
       </c>
       <c r="AB5" s="0">
-        <v>0.00029623454525024142</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="0">
-        <v>-0.00024388392117452844</v>
+        <v>-0.00023942405706511738</v>
       </c>
       <c r="AD5" s="0">
-        <v>4.3933754430753703e-05</v>
+        <v>4.333820007277135e-05</v>
       </c>
       <c r="AE5" s="0">
-        <v>0.00018134134161716946</v>
+        <v>0.00021084948019903647</v>
       </c>
       <c r="AF5" s="0">
-        <v>0.011035156532554628</v>
+        <v>0</v>
       </c>
       <c r="AG5" s="0">
-        <v>0.0005064398021335239</v>
+        <v>0.00046664920963698526</v>
       </c>
       <c r="AH5" s="0">
-        <v>0.00015415263488390257</v>
+        <v>0.00012369757606806603</v>
       </c>
       <c r="AI5" s="0">
-        <v>0.0018446925826976985</v>
+        <v>0.0020386045302981343</v>
       </c>
       <c r="AJ5" s="0">
-        <v>-4.9371460808075236e-05</v>
+        <v>-3.4254602248871881e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
@@ -4089,109 +4089,109 @@
         <v>40</v>
       </c>
       <c r="B6" s="0">
-        <v>-4.7151305485786037e-05</v>
+        <v>0</v>
       </c>
       <c r="C6" s="0">
-        <v>-3.6394161586080133e-05</v>
+        <v>0</v>
       </c>
       <c r="D6" s="0">
-        <v>0.0017518927242140261</v>
+        <v>0</v>
       </c>
       <c r="E6" s="0">
-        <v>8.0687521408920755e-05</v>
+        <v>7.7678482644046173e-05</v>
       </c>
       <c r="F6" s="0">
-        <v>-2.162391436173676e-05</v>
+        <v>-4.862882989801028e-05</v>
       </c>
       <c r="G6" s="0">
-        <v>0.00070212721619439581</v>
+        <v>0.0010255426091446982</v>
       </c>
       <c r="H6" s="0">
-        <v>3.7956588446601397e-05</v>
+        <v>0</v>
       </c>
       <c r="I6" s="0">
-        <v>-2.0205616740218453e-05</v>
+        <v>-2.8346386953999427e-05</v>
       </c>
       <c r="J6" s="0">
-        <v>0.00061513950723810179</v>
+        <v>0.00060304739188767888</v>
       </c>
       <c r="K6" s="0">
-        <v>-1.0289241151565745e-05</v>
+        <v>-1.4174770986509295e-05</v>
       </c>
       <c r="L6" s="0">
-        <v>0.00029482512673259265</v>
+        <v>0.00030797208158858924</v>
       </c>
       <c r="M6" s="0">
-        <v>0.015189795932083994</v>
+        <v>0.017930026775253328</v>
       </c>
       <c r="N6" s="0">
-        <v>0.00039929569179975483</v>
+        <v>0.00038074307539783816</v>
       </c>
       <c r="O6" s="0">
-        <v>0.00116631736939778</v>
+        <v>0.0011430794642848159</v>
       </c>
       <c r="P6" s="0">
-        <v>0.0059836774611622895</v>
+        <v>0.0058734236451490496</v>
       </c>
       <c r="Q6" s="0">
-        <v>6.6549508078336472e-05</v>
+        <v>0</v>
       </c>
       <c r="R6" s="0">
-        <v>6.1441816446559228e-05</v>
+        <v>0</v>
       </c>
       <c r="S6" s="0">
-        <v>0.00015204184402965398</v>
+        <v>0</v>
       </c>
       <c r="T6" s="0">
-        <v>0.00049343020661091479</v>
+        <v>0</v>
       </c>
       <c r="U6" s="0">
-        <v>1.5867539743170127e-05</v>
+        <v>1.6204515107630361e-05</v>
       </c>
       <c r="V6" s="0">
-        <v>-4.4279256951589191e-05</v>
+        <v>-4.336398510950368e-05</v>
       </c>
       <c r="W6" s="0">
-        <v>0.00016130864370395253</v>
+        <v>0.00018355129289014311</v>
       </c>
       <c r="X6" s="0">
-        <v>0.00038697370599768716</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="0">
-        <v>-3.6584887125359162e-05</v>
+        <v>-4.619771505310421e-05</v>
       </c>
       <c r="Z6" s="0">
-        <v>3.9891067432036566e-05</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="0">
-        <v>0.00080256574545762291</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="0">
-        <v>0.00010419015000716002</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="0">
-        <v>-4.1323314449312269e-05</v>
+        <v>-4.726062530257934e-05</v>
       </c>
       <c r="AD6" s="0">
-        <v>7.2679472901440717e-05</v>
+        <v>7.100494097926151e-05</v>
       </c>
       <c r="AE6" s="0">
-        <v>7.2880339802063163e-05</v>
+        <v>7.6018966679676332e-05</v>
       </c>
       <c r="AF6" s="0">
-        <v>0.0029805356660218257</v>
+        <v>0</v>
       </c>
       <c r="AG6" s="0">
-        <v>0.00011386289920508552</v>
+        <v>0.00012442663010070492</v>
       </c>
       <c r="AH6" s="0">
-        <v>-0.00014514714849990967</v>
+        <v>-0.00013464249782210849</v>
       </c>
       <c r="AI6" s="0">
-        <v>0.00029188859644743259</v>
+        <v>0.00034097477212365133</v>
       </c>
       <c r="AJ6" s="0">
-        <v>0.0041609284868505065</v>
+        <v>0.0039843550840720481</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
@@ -4199,109 +4199,109 @@
         <v>41</v>
       </c>
       <c r="B7" s="0">
-        <v>-4.1549667181313321e-05</v>
+        <v>0</v>
       </c>
       <c r="C7" s="0">
-        <v>-2.5046767268023781e-05</v>
+        <v>0</v>
       </c>
       <c r="D7" s="0">
-        <v>-7.6445208029103184e-05</v>
+        <v>0</v>
       </c>
       <c r="E7" s="0">
-        <v>9.2535663395978017e-06</v>
+        <v>1.2090456162498438e-05</v>
       </c>
       <c r="F7" s="0">
-        <v>-6.4388905678286749e-06</v>
+        <v>0</v>
       </c>
       <c r="G7" s="0">
-        <v>0.00042896677628293499</v>
+        <v>0</v>
       </c>
       <c r="H7" s="0">
-        <v>-5.0020194386298032e-05</v>
+        <v>0</v>
       </c>
       <c r="I7" s="0">
-        <v>1.782044238346544e-05</v>
+        <v>1.5869540735397726e-05</v>
       </c>
       <c r="J7" s="0">
-        <v>6.8638829035037982e-05</v>
+        <v>9.0544412407530454e-05</v>
       </c>
       <c r="K7" s="0">
-        <v>-3.1430768643361551e-06</v>
+        <v>-3.4845176731312947e-06</v>
       </c>
       <c r="L7" s="0">
-        <v>0.00045551202909504396</v>
+        <v>0.00044443835618308565</v>
       </c>
       <c r="M7" s="0">
-        <v>0.00091061889749326729</v>
+        <v>0.0015580198686684448</v>
       </c>
       <c r="N7" s="0">
-        <v>0.00014963764452774112</v>
+        <v>0.0001581319970575662</v>
       </c>
       <c r="O7" s="0">
-        <v>0.0032327907451164049</v>
+        <v>0.0031118602070678574</v>
       </c>
       <c r="P7" s="0">
-        <v>0.12040703003971563</v>
+        <v>0.11435015515080384</v>
       </c>
       <c r="Q7" s="0">
-        <v>-2.5428130643292694e-05</v>
+        <v>0</v>
       </c>
       <c r="R7" s="0">
-        <v>-7.2237424711001549e-05</v>
+        <v>0</v>
       </c>
       <c r="S7" s="0">
-        <v>8.5694963319519498e-07</v>
+        <v>0</v>
       </c>
       <c r="T7" s="0">
-        <v>2.8519148802421935e-05</v>
+        <v>0</v>
       </c>
       <c r="U7" s="0">
-        <v>4.9979096033229692e-05</v>
+        <v>4.8042121421566708e-05</v>
       </c>
       <c r="V7" s="0">
-        <v>9.7285256591940405e-05</v>
+        <v>9.0568069187039403e-05</v>
       </c>
       <c r="W7" s="0">
-        <v>0.00011328386573444669</v>
+        <v>0.00011893198331798023</v>
       </c>
       <c r="X7" s="0">
-        <v>0.00063502398761189067</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="0">
-        <v>1.9992985841916979e-05</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="0">
-        <v>6.4546616330540528e-06</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="0">
-        <v>0.00030919911740227206</v>
+        <v>0</v>
       </c>
       <c r="AB7" s="0">
-        <v>6.8542688890911718e-05</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="0">
-        <v>1.372461742071101e-05</v>
+        <v>1.1147846380654419e-05</v>
       </c>
       <c r="AD7" s="0">
-        <v>5.3474339475949384e-06</v>
+        <v>0</v>
       </c>
       <c r="AE7" s="0">
-        <v>6.0235677367021125e-05</v>
+        <v>0</v>
       </c>
       <c r="AF7" s="0">
-        <v>0.0014842923312444018</v>
+        <v>0</v>
       </c>
       <c r="AG7" s="0">
-        <v>-0.00038843093378439155</v>
+        <v>-0.0003631035255450763</v>
       </c>
       <c r="AH7" s="0">
-        <v>-3.2697062588589614e-05</v>
+        <v>-3.6835680250568855e-05</v>
       </c>
       <c r="AI7" s="0">
-        <v>-0.0011066356942764459</v>
+        <v>-0.0010354096825807078</v>
       </c>
       <c r="AJ7" s="0">
-        <v>0.0079825859110482424</v>
+        <v>0.007735117025939999</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
@@ -4309,109 +4309,109 @@
         <v>42</v>
       </c>
       <c r="B8" s="0">
-        <v>-1.5208904781074592e-05</v>
+        <v>0</v>
       </c>
       <c r="C8" s="0">
-        <v>-1.6135233314136777e-06</v>
+        <v>0</v>
       </c>
       <c r="D8" s="0">
-        <v>-7.2455521687759218e-05</v>
+        <v>0</v>
       </c>
       <c r="E8" s="0">
-        <v>-6.6888362382865502e-06</v>
+        <v>0</v>
       </c>
       <c r="F8" s="0">
-        <v>-8.7681086354626863e-07</v>
+        <v>0</v>
       </c>
       <c r="G8" s="0">
-        <v>1.5844261402993861e-05</v>
+        <v>0</v>
       </c>
       <c r="H8" s="0">
-        <v>-4.4578708435251698e-05</v>
+        <v>0</v>
       </c>
       <c r="I8" s="0">
-        <v>4.1826418793114493e-06</v>
+        <v>0</v>
       </c>
       <c r="J8" s="0">
-        <v>6.7931893671912823e-05</v>
+        <v>0</v>
       </c>
       <c r="K8" s="0">
-        <v>-1.0590728428169864e-05</v>
+        <v>0</v>
       </c>
       <c r="L8" s="0">
-        <v>6.2191890824098774e-05</v>
+        <v>0</v>
       </c>
       <c r="M8" s="0">
-        <v>0.00011978546192602567</v>
+        <v>0.00017641354760972988</v>
       </c>
       <c r="N8" s="0">
-        <v>1.7003969085020048e-05</v>
+        <v>2.3964656536809344e-05</v>
       </c>
       <c r="O8" s="0">
-        <v>0.002628728279572899</v>
+        <v>0.0026296002893639345</v>
       </c>
       <c r="P8" s="0">
-        <v>-0.032236489955994291</v>
+        <v>-0.024110440966529097</v>
       </c>
       <c r="Q8" s="0">
-        <v>2.3832993862682162e-06</v>
+        <v>0</v>
       </c>
       <c r="R8" s="0">
-        <v>-0.00015337892075196558</v>
+        <v>0</v>
       </c>
       <c r="S8" s="0">
-        <v>-3.3519421631817725e-05</v>
+        <v>0</v>
       </c>
       <c r="T8" s="0">
-        <v>-0.00010763345370111317</v>
+        <v>0</v>
       </c>
       <c r="U8" s="0">
-        <v>2.6760042673895875e-05</v>
+        <v>2.7642740027601441e-05</v>
       </c>
       <c r="V8" s="0">
-        <v>0.00012776487247848458</v>
+        <v>0.00012495203460922993</v>
       </c>
       <c r="W8" s="0">
-        <v>4.0535091551938201e-05</v>
+        <v>4.5658329325754061e-05</v>
       </c>
       <c r="X8" s="0">
-        <v>-0.00023702417520384068</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="0">
-        <v>5.9963843760893281e-06</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="0">
-        <v>2.0514579070382577e-05</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="0">
-        <v>3.7102019900648453e-06</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="0">
-        <v>-7.553431705585798e-05</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="0">
-        <v>-1.6361246823355977e-06</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="0">
-        <v>4.2775101721465184e-05</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="0">
-        <v>9.5941455958229684e-06</v>
+        <v>0</v>
       </c>
       <c r="AF8" s="0">
-        <v>-0.00092616085304957302</v>
+        <v>0</v>
       </c>
       <c r="AG8" s="0">
-        <v>0.00011245724242672947</v>
+        <v>8.5868966087145719e-05</v>
       </c>
       <c r="AH8" s="0">
-        <v>0.00019242125514585978</v>
+        <v>0.00017856335368775055</v>
       </c>
       <c r="AI8" s="0">
-        <v>0.00018846799554967232</v>
+        <v>0.00012092289941656274</v>
       </c>
       <c r="AJ8" s="0">
-        <v>-0.0025496085658574248</v>
+        <v>-0.0019809737804309482</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
@@ -4419,109 +4419,109 @@
         <v>43</v>
       </c>
       <c r="B9" s="0">
-        <v>5.6494393729769709e-06</v>
+        <v>0</v>
       </c>
       <c r="C9" s="0">
-        <v>2.9568056534472527e-06</v>
+        <v>0</v>
       </c>
       <c r="D9" s="0">
-        <v>7.383012730959954e-06</v>
+        <v>0</v>
       </c>
       <c r="E9" s="0">
-        <v>1.5219747012552159e-05</v>
+        <v>0</v>
       </c>
       <c r="F9" s="0">
-        <v>1.9377417927266891e-06</v>
+        <v>0</v>
       </c>
       <c r="G9" s="0">
-        <v>6.1340756283732409e-05</v>
+        <v>0</v>
       </c>
       <c r="H9" s="0">
-        <v>1.2104491672616034e-05</v>
+        <v>0</v>
       </c>
       <c r="I9" s="0">
-        <v>0.00012564421892818976</v>
+        <v>0</v>
       </c>
       <c r="J9" s="0">
-        <v>0.00021133429308166311</v>
+        <v>0</v>
       </c>
       <c r="K9" s="0">
-        <v>2.0526890195833896e-06</v>
+        <v>0</v>
       </c>
       <c r="L9" s="0">
-        <v>0.00027578124240489141</v>
+        <v>0</v>
       </c>
       <c r="M9" s="0">
-        <v>4.440420635799174e-05</v>
+        <v>5.0251897457094734e-05</v>
       </c>
       <c r="N9" s="0">
-        <v>0.00020285833913778691</v>
+        <v>0.00018941967143387719</v>
       </c>
       <c r="O9" s="0">
-        <v>0.00028574302683952895</v>
+        <v>0.0004285197817623502</v>
       </c>
       <c r="P9" s="0">
-        <v>-0.0039443325429986548</v>
+        <v>-0.0054023464231868993</v>
       </c>
       <c r="Q9" s="0">
-        <v>-2.0278051704392352e-05</v>
+        <v>0</v>
       </c>
       <c r="R9" s="0">
-        <v>4.3137996973482567e-05</v>
+        <v>0</v>
       </c>
       <c r="S9" s="0">
-        <v>5.0123052425364662e-06</v>
+        <v>0</v>
       </c>
       <c r="T9" s="0">
-        <v>1.1864042923813189e-05</v>
+        <v>0</v>
       </c>
       <c r="U9" s="0">
-        <v>1.951381192011581e-05</v>
+        <v>1.9793285574498207e-05</v>
       </c>
       <c r="V9" s="0">
-        <v>8.8384862260082297e-06</v>
+        <v>1.6081756315777398e-05</v>
       </c>
       <c r="W9" s="0">
-        <v>3.0328512416080502e-05</v>
+        <v>3.1966701977480259e-05</v>
       </c>
       <c r="X9" s="0">
-        <v>-1.1644421512543643e-05</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="0">
-        <v>1.1284214873023038e-05</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="0">
-        <v>-4.109020258806495e-05</v>
+        <v>0</v>
       </c>
       <c r="AA9" s="0">
-        <v>-8.1139124899152405e-05</v>
+        <v>0</v>
       </c>
       <c r="AB9" s="0">
-        <v>6.9438816083361263e-06</v>
+        <v>0</v>
       </c>
       <c r="AC9" s="0">
-        <v>1.5926039475691236e-06</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="0">
-        <v>9.2806430309540677e-05</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="0">
-        <v>6.2581539778242166e-05</v>
+        <v>0</v>
       </c>
       <c r="AF9" s="0">
-        <v>3.9134310713528691e-06</v>
+        <v>0</v>
       </c>
       <c r="AG9" s="0">
-        <v>-2.3419113961695577e-05</v>
+        <v>-1.5581796763211163e-05</v>
       </c>
       <c r="AH9" s="0">
-        <v>2.3018775091016288e-05</v>
+        <v>3.2870931759594714e-05</v>
       </c>
       <c r="AI9" s="0">
-        <v>4.5925326435168709e-05</v>
+        <v>5.2142414497093688e-05</v>
       </c>
       <c r="AJ9" s="0">
-        <v>-0.00022063395383071762</v>
+        <v>-0.00034499437963450471</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
@@ -4529,109 +4529,109 @@
         <v>44</v>
       </c>
       <c r="B10" s="0">
-        <v>7.3036740525585314e-07</v>
+        <v>0</v>
       </c>
       <c r="C10" s="0">
-        <v>-7.4941111776878874e-08</v>
+        <v>0</v>
       </c>
       <c r="D10" s="0">
-        <v>2.0025265715898884e-06</v>
+        <v>0</v>
       </c>
       <c r="E10" s="0">
-        <v>2.6559877770284964e-06</v>
+        <v>0</v>
       </c>
       <c r="F10" s="0">
-        <v>-8.6889849119000996e-08</v>
+        <v>0</v>
       </c>
       <c r="G10" s="0">
-        <v>-1.3017358541715944e-05</v>
+        <v>0</v>
       </c>
       <c r="H10" s="0">
-        <v>1.8881044013917167e-06</v>
+        <v>0</v>
       </c>
       <c r="I10" s="0">
-        <v>0.00017825639580331117</v>
+        <v>0</v>
       </c>
       <c r="J10" s="0">
-        <v>2.2077763184956423e-05</v>
+        <v>0</v>
       </c>
       <c r="K10" s="0">
-        <v>5.72086514552538e-07</v>
+        <v>0</v>
       </c>
       <c r="L10" s="0">
-        <v>1.4011736916504294e-05</v>
+        <v>0</v>
       </c>
       <c r="M10" s="0">
-        <v>4.1921492483334909e-05</v>
+        <v>4.1863167523402162e-05</v>
       </c>
       <c r="N10" s="0">
-        <v>-5.346990946836619e-05</v>
+        <v>-3.4924153522744559e-05</v>
       </c>
       <c r="O10" s="0">
-        <v>-0.00018096894410085654</v>
+        <v>-0.00014013916843144854</v>
       </c>
       <c r="P10" s="0">
-        <v>0.0022050612677944215</v>
+        <v>0.0016814616308938113</v>
       </c>
       <c r="Q10" s="0">
-        <v>5.1780065604991644e-06</v>
+        <v>0</v>
       </c>
       <c r="R10" s="0">
-        <v>1.0031314415493379e-05</v>
+        <v>0</v>
       </c>
       <c r="S10" s="0">
-        <v>1.5280741218796834e-06</v>
+        <v>0</v>
       </c>
       <c r="T10" s="0">
-        <v>5.5061422662559991e-06</v>
+        <v>0</v>
       </c>
       <c r="U10" s="0">
-        <v>-9.9918265554738841e-06</v>
+        <v>-7.750997485578599e-06</v>
       </c>
       <c r="V10" s="0">
-        <v>0.00010582417456995053</v>
+        <v>9.8231602622660447e-05</v>
       </c>
       <c r="W10" s="0">
-        <v>0.00022204410123893953</v>
+        <v>0.00021403991955625811</v>
       </c>
       <c r="X10" s="0">
-        <v>1.4869319943924279e-05</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="0">
-        <v>-1.0333700916501811e-05</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="0">
-        <v>7.3719572834004256e-06</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="0">
-        <v>9.980583548944749e-06</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="0">
-        <v>4.0837806445019833e-06</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="0">
-        <v>2.9727964714054558e-06</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="0">
-        <v>-4.3543810031075425e-05</v>
+        <v>0</v>
       </c>
       <c r="AE10" s="0">
-        <v>-2.056213583868333e-05</v>
+        <v>0</v>
       </c>
       <c r="AF10" s="0">
-        <v>5.4909274980523309e-05</v>
+        <v>0</v>
       </c>
       <c r="AG10" s="0">
-        <v>0.00024774664426160616</v>
+        <v>0.00022593598518533029</v>
       </c>
       <c r="AH10" s="0">
-        <v>-4.3807178238573961e-05</v>
+        <v>-3.8160151754628768e-05</v>
       </c>
       <c r="AI10" s="0">
-        <v>2.4581104093688324e-05</v>
+        <v>2.612378316144149e-05</v>
       </c>
       <c r="AJ10" s="0">
-        <v>0.00016624615443087032</v>
+        <v>0.00013178975761330087</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
@@ -4639,109 +4639,109 @@
         <v>45</v>
       </c>
       <c r="B11" s="0">
-        <v>-3.7127065893167009e-07</v>
+        <v>0</v>
       </c>
       <c r="C11" s="0">
-        <v>-1.645042103600354e-07</v>
+        <v>0</v>
       </c>
       <c r="D11" s="0">
-        <v>-3.4724144989317384e-07</v>
+        <v>0</v>
       </c>
       <c r="E11" s="0">
-        <v>-2.127231780322284e-06</v>
+        <v>0</v>
       </c>
       <c r="F11" s="0">
-        <v>-1.163412738944146e-07</v>
+        <v>0</v>
       </c>
       <c r="G11" s="0">
-        <v>-7.9002358437015536e-07</v>
+        <v>0</v>
       </c>
       <c r="H11" s="0">
-        <v>-8.2811004696334061e-07</v>
+        <v>0</v>
       </c>
       <c r="I11" s="0">
-        <v>-5.7060111515591018e-05</v>
+        <v>0</v>
       </c>
       <c r="J11" s="0">
-        <v>-1.4257392949445612e-05</v>
+        <v>0</v>
       </c>
       <c r="K11" s="0">
-        <v>-1.634067422085998e-07</v>
+        <v>0</v>
       </c>
       <c r="L11" s="0">
-        <v>-1.594455607932268e-05</v>
+        <v>0</v>
       </c>
       <c r="M11" s="0">
-        <v>-2.6607225951894234e-05</v>
+        <v>-2.0718717936623722e-05</v>
       </c>
       <c r="N11" s="0">
-        <v>-7.054634562312152e-06</v>
+        <v>-9.99886740890484e-06</v>
       </c>
       <c r="O11" s="0">
-        <v>4.9231969104145682e-06</v>
+        <v>-8.7231907416709009e-06</v>
       </c>
       <c r="P11" s="0">
-        <v>2.4439615888103901e-05</v>
+        <v>0.00018167696331588686</v>
       </c>
       <c r="Q11" s="0">
-        <v>1.395363206881122e-06</v>
+        <v>0</v>
       </c>
       <c r="R11" s="0">
-        <v>-4.3536567041328749e-06</v>
+        <v>0</v>
       </c>
       <c r="S11" s="0">
-        <v>-3.8701849630683343e-07</v>
+        <v>0</v>
       </c>
       <c r="T11" s="0">
-        <v>-1.0530003652663034e-06</v>
+        <v>0</v>
       </c>
       <c r="U11" s="0">
-        <v>2.6882338245364753e-08</v>
+        <v>-7.0067980603305147e-07</v>
       </c>
       <c r="V11" s="0">
-        <v>-2.238699988048288e-05</v>
+        <v>0</v>
       </c>
       <c r="W11" s="0">
-        <v>0.0001697059981174469</v>
+        <v>0</v>
       </c>
       <c r="X11" s="0">
-        <v>-6.1112827447396187e-07</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="0">
-        <v>1.0202020551196702e-06</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="0">
-        <v>2.9854569024311942e-06</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="0">
-        <v>4.1488107395757911e-06</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="0">
-        <v>-7.2011227288782165e-07</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="0">
-        <v>-1.7605316731764651e-06</v>
+        <v>0</v>
       </c>
       <c r="AD11" s="0">
-        <v>-1.8084498700230647e-06</v>
+        <v>0</v>
       </c>
       <c r="AE11" s="0">
-        <v>-1.3500844730500638e-06</v>
+        <v>0</v>
       </c>
       <c r="AF11" s="0">
-        <v>-4.3806166092014003e-06</v>
+        <v>0</v>
       </c>
       <c r="AG11" s="0">
-        <v>-9.9544879009559809e-05</v>
+        <v>-7.0965866965837414e-05</v>
       </c>
       <c r="AH11" s="0">
-        <v>5.0194947910372612e-06</v>
+        <v>1.1963105765794895e-06</v>
       </c>
       <c r="AI11" s="0">
-        <v>-1.3801222049553014e-05</v>
+        <v>-1.0449081217817674e-05</v>
       </c>
       <c r="AJ11" s="0">
-        <v>-1.862101896489793e-06</v>
+        <v>1.0553925057962015e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
@@ -4749,109 +4749,109 @@
         <v>46</v>
       </c>
       <c r="B12" s="0">
-        <v>-1.5366826247485867e-08</v>
+        <v>0</v>
       </c>
       <c r="C12" s="0">
-        <v>1.3663201496813855e-08</v>
+        <v>0</v>
       </c>
       <c r="D12" s="0">
-        <v>-4.94398097382036e-08</v>
+        <v>0</v>
       </c>
       <c r="E12" s="0">
-        <v>3.5697297154333199e-08</v>
+        <v>0</v>
       </c>
       <c r="F12" s="0">
-        <v>1.2256909925337255e-08</v>
+        <v>0</v>
       </c>
       <c r="G12" s="0">
-        <v>4.4820298938971805e-07</v>
+        <v>0</v>
       </c>
       <c r="H12" s="0">
-        <v>-3.8353917195246723e-08</v>
+        <v>0</v>
       </c>
       <c r="I12" s="0">
-        <v>-4.9971958285211572e-06</v>
+        <v>0</v>
       </c>
       <c r="J12" s="0">
-        <v>4.3703737708920857e-07</v>
+        <v>0</v>
       </c>
       <c r="K12" s="0">
-        <v>-1.8252323338416632e-08</v>
+        <v>0</v>
       </c>
       <c r="L12" s="0">
-        <v>8.0160856745331904e-07</v>
+        <v>0</v>
       </c>
       <c r="M12" s="0">
-        <v>6.4209810815481293e-07</v>
+        <v>-1.5862432918893907e-06</v>
       </c>
       <c r="N12" s="0">
-        <v>3.6669486702491147e-06</v>
+        <v>2.4934572952848006e-06</v>
       </c>
       <c r="O12" s="0">
-        <v>5.5589542308012608e-06</v>
+        <v>4.7693518353950404e-06</v>
       </c>
       <c r="P12" s="0">
-        <v>-0.00010628476401837095</v>
+        <v>-8.5393561441663181e-05</v>
       </c>
       <c r="Q12" s="0">
-        <v>-5.725947866611563e-07</v>
+        <v>0</v>
       </c>
       <c r="R12" s="0">
-        <v>-3.020186743622544e-07</v>
+        <v>0</v>
       </c>
       <c r="S12" s="0">
-        <v>-4.6537338208073674e-08</v>
+        <v>0</v>
       </c>
       <c r="T12" s="0">
-        <v>-1.9561307435702838e-07</v>
+        <v>0</v>
       </c>
       <c r="U12" s="0">
-        <v>5.7456926443040515e-07</v>
+        <v>0</v>
       </c>
       <c r="V12" s="0">
-        <v>0.002444195739442467</v>
+        <v>0</v>
       </c>
       <c r="W12" s="0">
-        <v>0.0041964790709907536</v>
+        <v>0</v>
       </c>
       <c r="X12" s="0">
-        <v>-6.6668239946137144e-07</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="0">
-        <v>8.0969370341555201e-07</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="0">
-        <v>-9.0869849788306534e-07</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="0">
-        <v>-8.4412821991691377e-07</v>
+        <v>0</v>
       </c>
       <c r="AB12" s="0">
-        <v>-1.4977041912785741e-07</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="0">
-        <v>4.8413774155958095e-08</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="0">
-        <v>3.8094448130385939e-06</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="0">
-        <v>1.3090347244199296e-06</v>
+        <v>0</v>
       </c>
       <c r="AF12" s="0">
-        <v>-2.3487452915600139e-06</v>
+        <v>0</v>
       </c>
       <c r="AG12" s="0">
-        <v>-4.5647014261321621e-06</v>
+        <v>-1.1866276149735345e-05</v>
       </c>
       <c r="AH12" s="0">
-        <v>0.0026779272422457799</v>
+        <v>0.0024048714468788883</v>
       </c>
       <c r="AI12" s="0">
-        <v>0.00099960470875918358</v>
+        <v>0.0008965240195439705</v>
       </c>
       <c r="AJ12" s="0">
-        <v>-7.764037625112658e-06</v>
+        <v>-6.5311064690464815e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
@@ -4859,109 +4859,109 @@
         <v>47</v>
       </c>
       <c r="B13" s="0">
-        <v>1.8567144231054884e-08</v>
+        <v>0</v>
       </c>
       <c r="C13" s="0">
-        <v>6.9924083048526808e-09</v>
+        <v>0</v>
       </c>
       <c r="D13" s="0">
-        <v>1.4134331065558698e-08</v>
+        <v>0</v>
       </c>
       <c r="E13" s="0">
-        <v>1.1767667125175953e-07</v>
+        <v>0</v>
       </c>
       <c r="F13" s="0">
-        <v>4.968567937282329e-09</v>
+        <v>0</v>
       </c>
       <c r="G13" s="0">
-        <v>4.7037252321971661e-09</v>
+        <v>0</v>
       </c>
       <c r="H13" s="0">
-        <v>4.1502566653824022e-08</v>
+        <v>0</v>
       </c>
       <c r="I13" s="0">
-        <v>3.6513886785794003e-06</v>
+        <v>0</v>
       </c>
       <c r="J13" s="0">
-        <v>4.3193272128278169e-07</v>
+        <v>0</v>
       </c>
       <c r="K13" s="0">
-        <v>8.9696268892556638e-09</v>
+        <v>0</v>
       </c>
       <c r="L13" s="0">
-        <v>4.6913510299856492e-07</v>
+        <v>0</v>
       </c>
       <c r="M13" s="0">
-        <v>1.5782638761393115e-06</v>
+        <v>1.3451655537511411e-06</v>
       </c>
       <c r="N13" s="0">
-        <v>7.3873738672439293e-08</v>
+        <v>3.7828931251300998e-07</v>
       </c>
       <c r="O13" s="0">
-        <v>-4.3778893353532323e-07</v>
+        <v>0</v>
       </c>
       <c r="P13" s="0">
-        <v>6.0222808722403303e-06</v>
+        <v>-4.4617620386685393e-06</v>
       </c>
       <c r="Q13" s="0">
-        <v>-4.310569574110132e-08</v>
+        <v>0</v>
       </c>
       <c r="R13" s="0">
-        <v>2.8600971727673539e-07</v>
+        <v>0</v>
       </c>
       <c r="S13" s="0">
-        <v>2.0828467977764005e-08</v>
+        <v>0</v>
       </c>
       <c r="T13" s="0">
-        <v>6.1082070357708558e-08</v>
+        <v>0</v>
       </c>
       <c r="U13" s="0">
-        <v>-4.7768446589569035e-08</v>
+        <v>0</v>
       </c>
       <c r="V13" s="0">
-        <v>0.00020706991443365886</v>
+        <v>0</v>
       </c>
       <c r="W13" s="0">
-        <v>0.042628745240757694</v>
+        <v>0</v>
       </c>
       <c r="X13" s="0">
-        <v>7.2727963887760633e-08</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="0">
-        <v>-1.7173441059487756e-07</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="0">
-        <v>-1.1544378760018611e-07</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="0">
-        <v>-1.4574571614523165e-07</v>
+        <v>0</v>
       </c>
       <c r="AB13" s="0">
-        <v>4.3629014571111711e-08</v>
+        <v>0</v>
       </c>
       <c r="AC13" s="0">
-        <v>1.4367700676034989e-07</v>
+        <v>0</v>
       </c>
       <c r="AD13" s="0">
-        <v>-2.8003026765920547e-07</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="0">
-        <v>-3.8999610129018523e-08</v>
+        <v>0</v>
       </c>
       <c r="AF13" s="0">
-        <v>3.5216669137914505e-07</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="0">
-        <v>3.936151408269144e-05</v>
+        <v>3.4099178048161724e-05</v>
       </c>
       <c r="AH13" s="0">
-        <v>0.00064970270463956799</v>
+        <v>0.00083445580974007957</v>
       </c>
       <c r="AI13" s="0">
-        <v>0.00024984076780212692</v>
+        <v>0.00031793896934245746</v>
       </c>
       <c r="AJ13" s="0">
-        <v>6.0032451804831444e-07</v>
+        <v>-1.9962398763865278e-07</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
@@ -4969,109 +4969,109 @@
         <v>48</v>
       </c>
       <c r="B14" s="0">
-        <v>-3.7317005643725341e-10</v>
+        <v>0</v>
       </c>
       <c r="C14" s="0">
-        <v>-1.0168663691375635e-09</v>
+        <v>0</v>
       </c>
       <c r="D14" s="0">
-        <v>9.3711122242737551e-10</v>
+        <v>0</v>
       </c>
       <c r="E14" s="0">
-        <v>-1.0219770593713774e-08</v>
+        <v>0</v>
       </c>
       <c r="F14" s="0">
-        <v>-8.6387321028509076e-10</v>
+        <v>0</v>
       </c>
       <c r="G14" s="0">
-        <v>-1.5273160286365268e-08</v>
+        <v>0</v>
       </c>
       <c r="H14" s="0">
-        <v>-8.4912866999898382e-10</v>
+        <v>0</v>
       </c>
       <c r="I14" s="0">
-        <v>-2.7077105356566194e-08</v>
+        <v>0</v>
       </c>
       <c r="J14" s="0">
-        <v>-3.5629229818979982e-08</v>
+        <v>0</v>
       </c>
       <c r="K14" s="0">
-        <v>2.7263618059441172e-10</v>
+        <v>0</v>
       </c>
       <c r="L14" s="0">
-        <v>-4.9683703237511107e-08</v>
+        <v>0</v>
       </c>
       <c r="M14" s="0">
-        <v>-1.6247261068827128e-07</v>
+        <v>2.1152546728277481e-08</v>
       </c>
       <c r="N14" s="0">
-        <v>-1.7861407816381035e-07</v>
+        <v>-1.3001698598877032e-07</v>
       </c>
       <c r="O14" s="0">
-        <v>-1.6413313173746416e-07</v>
+        <v>0</v>
       </c>
       <c r="P14" s="0">
-        <v>4.2239720803714554e-06</v>
+        <v>3.7541085627019723e-06</v>
       </c>
       <c r="Q14" s="0">
-        <v>3.8719383732334942e-08</v>
+        <v>0</v>
       </c>
       <c r="R14" s="0">
-        <v>-3.8631224557438393e-09</v>
+        <v>0</v>
       </c>
       <c r="S14" s="0">
-        <v>7.2351498159426135e-10</v>
+        <v>0</v>
       </c>
       <c r="T14" s="0">
-        <v>4.8063856735666824e-09</v>
+        <v>0</v>
       </c>
       <c r="U14" s="0">
-        <v>0.00013312015085017802</v>
+        <v>0</v>
       </c>
       <c r="V14" s="0">
-        <v>-0.00031659452776612037</v>
+        <v>0</v>
       </c>
       <c r="W14" s="0">
-        <v>-0.0091552425960765103</v>
+        <v>0</v>
       </c>
       <c r="X14" s="0">
-        <v>2.4381150047174478e-08</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="0">
-        <v>-3.6626829115444889e-08</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="0">
-        <v>6.4601452720356651e-08</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="0">
-        <v>4.8214498103609895e-08</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="0">
-        <v>3.8537829780620936e-09</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="0">
-        <v>-2.0161820822313969e-08</v>
+        <v>0</v>
       </c>
       <c r="AD14" s="0">
-        <v>-2.1042193338664695e-07</v>
+        <v>0</v>
       </c>
       <c r="AE14" s="0">
-        <v>-5.9436743271008548e-08</v>
+        <v>0</v>
       </c>
       <c r="AF14" s="0">
-        <v>8.0896351961405835e-08</v>
+        <v>0</v>
       </c>
       <c r="AG14" s="0">
-        <v>0.00029458633690905762</v>
+        <v>0.00026299211136511139</v>
       </c>
       <c r="AH14" s="0">
-        <v>-0.00074236136409213153</v>
+        <v>-0.00056932862564710695</v>
       </c>
       <c r="AI14" s="0">
-        <v>-0.00020052953013685099</v>
+        <v>-0.00014446628823431648</v>
       </c>
       <c r="AJ14" s="0">
-        <v>2.9887720382256641e-07</v>
+        <v>2.8185373561097534e-07</v>
       </c>
     </row>
   </sheetData>
@@ -5085,37 +5085,37 @@
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="true"/>
-    <col min="2" max="2" width="15.5703125" customWidth="true"/>
+    <col min="2" max="2" width="15.7109375" customWidth="true"/>
     <col min="3" max="3" width="15.7109375" customWidth="true"/>
-    <col min="4" max="4" width="15.5703125" customWidth="true"/>
+    <col min="4" max="4" width="14.7109375" customWidth="true"/>
     <col min="5" max="5" width="15.5703125" customWidth="true"/>
-    <col min="6" max="6" width="15.5703125" customWidth="true"/>
-    <col min="7" max="7" width="15.7109375" customWidth="true"/>
-    <col min="8" max="8" width="15.5703125" customWidth="true"/>
+    <col min="6" max="6" width="14.7109375" customWidth="true"/>
+    <col min="7" max="7" width="14.7109375" customWidth="true"/>
+    <col min="8" max="8" width="13.7109375" customWidth="true"/>
     <col min="9" max="9" width="15.7109375" customWidth="true"/>
     <col min="10" max="10" width="15.7109375" customWidth="true"/>
-    <col min="11" max="11" width="15.5703125" customWidth="true"/>
+    <col min="11" max="11" width="13.7109375" customWidth="true"/>
     <col min="12" max="12" width="15.7109375" customWidth="true"/>
     <col min="13" max="13" width="15.7109375" customWidth="true"/>
     <col min="14" max="14" width="15.7109375" customWidth="true"/>
     <col min="15" max="15" width="15.7109375" customWidth="true"/>
-    <col min="16" max="16" width="15.5703125" customWidth="true"/>
-    <col min="17" max="17" width="15.5703125" customWidth="true"/>
+    <col min="16" max="16" width="16.28515625" customWidth="true"/>
+    <col min="17" max="17" width="14.7109375" customWidth="true"/>
     <col min="18" max="18" width="15.7109375" customWidth="true"/>
-    <col min="19" max="19" width="15.7109375" customWidth="true"/>
-    <col min="20" max="20" width="15.7109375" customWidth="true"/>
+    <col min="19" max="19" width="7" customWidth="true"/>
+    <col min="20" max="20" width="14.7109375" customWidth="true"/>
     <col min="21" max="21" width="15.5703125" customWidth="true"/>
     <col min="22" max="22" width="15.7109375" customWidth="true"/>
     <col min="23" max="23" width="15.7109375" customWidth="true"/>
-    <col min="24" max="24" width="15.7109375" customWidth="true"/>
-    <col min="25" max="25" width="15.7109375" customWidth="true"/>
-    <col min="26" max="26" width="15.5703125" customWidth="true"/>
-    <col min="27" max="27" width="15.7109375" customWidth="true"/>
-    <col min="28" max="28" width="15.7109375" customWidth="true"/>
-    <col min="29" max="29" width="15.5703125" customWidth="true"/>
+    <col min="24" max="24" width="14.7109375" customWidth="true"/>
+    <col min="25" max="25" width="14.7109375" customWidth="true"/>
+    <col min="26" max="26" width="13.7109375" customWidth="true"/>
+    <col min="27" max="27" width="14.7109375" customWidth="true"/>
+    <col min="28" max="28" width="13.7109375" customWidth="true"/>
+    <col min="29" max="29" width="15.7109375" customWidth="true"/>
     <col min="30" max="30" width="15.5703125" customWidth="true"/>
     <col min="31" max="31" width="15.7109375" customWidth="true"/>
-    <col min="32" max="32" width="15.5703125" customWidth="true"/>
+    <col min="32" max="32" width="13.7109375" customWidth="true"/>
     <col min="33" max="33" width="15.7109375" customWidth="true"/>
     <col min="34" max="34" width="15.7109375" customWidth="true"/>
     <col min="35" max="35" width="15.7109375" customWidth="true"/>
@@ -5237,109 +5237,109 @@
         <v>36</v>
       </c>
       <c r="B2" s="0">
-        <v>0.8935047534745163</v>
+        <v>0.89376114819033725</v>
       </c>
       <c r="C2" s="0">
-        <v>0.99512810556936548</v>
+        <v>0.99514840557432582</v>
       </c>
       <c r="D2" s="0">
-        <v>0.94387694748388218</v>
+        <v>0.94746484268514786</v>
       </c>
       <c r="E2" s="0">
-        <v>0.89146338293409388</v>
+        <v>0.89254810491114367</v>
       </c>
       <c r="F2" s="0">
-        <v>0.98964254758468051</v>
+        <v>0.98968452493307979</v>
       </c>
       <c r="G2" s="0">
-        <v>0.97867228603761125</v>
+        <v>0.97920481428562911</v>
       </c>
       <c r="H2" s="0">
-        <v>0.90201061645880887</v>
+        <v>0.90302441025097868</v>
       </c>
       <c r="I2" s="0">
-        <v>0.99436555746417898</v>
+        <v>0.99468646797741123</v>
       </c>
       <c r="J2" s="0">
-        <v>0.9740438781895201</v>
+        <v>0.97434251081769352</v>
       </c>
       <c r="K2" s="0">
-        <v>0.9282376455203124</v>
+        <v>0.92895336025799236</v>
       </c>
       <c r="L2" s="0">
-        <v>0.92401187669929619</v>
+        <v>0.92436077059679789</v>
       </c>
       <c r="M2" s="0">
-        <v>0.82727857803992721</v>
+        <v>0.82781551862588831</v>
       </c>
       <c r="N2" s="0">
-        <v>0.94142029136977623</v>
+        <v>0.94145721499847757</v>
       </c>
       <c r="O2" s="0">
-        <v>0.98028676672376114</v>
+        <v>0.9803187910581026</v>
       </c>
       <c r="P2" s="0">
-        <v>0.70897761940434434</v>
+        <v>0.70897799349932367</v>
       </c>
       <c r="Q2" s="0">
-        <v>0.99715789009661937</v>
+        <v>0.99726265354537658</v>
       </c>
       <c r="R2" s="0">
-        <v>0.99957902589452607</v>
+        <v>0.9997376485500723</v>
       </c>
       <c r="S2" s="0">
-        <v>0.9995690841321675</v>
+        <v>1</v>
       </c>
       <c r="T2" s="0">
-        <v>0.99219360684525304</v>
+        <v>0.99333457561696192</v>
       </c>
       <c r="U2" s="0">
-        <v>0.98909577892724221</v>
+        <v>0.98935834866008154</v>
       </c>
       <c r="V2" s="0">
-        <v>0.99063508023952918</v>
+        <v>0.99334514446294253</v>
       </c>
       <c r="W2" s="0">
-        <v>0.94446031204194414</v>
+        <v>0.99060966912080828</v>
       </c>
       <c r="X2" s="0">
-        <v>0.9897785225420872</v>
+        <v>0.99099495944861993</v>
       </c>
       <c r="Y2" s="0">
-        <v>0.90122742942360579</v>
+        <v>0.90129149817926702</v>
       </c>
       <c r="Z2" s="0">
-        <v>0.93183024225314748</v>
+        <v>0.93258163193575505</v>
       </c>
       <c r="AA2" s="0">
-        <v>0.91865994549970653</v>
+        <v>0.91995500977575284</v>
       </c>
       <c r="AB2" s="0">
-        <v>0.96512659491158803</v>
+        <v>0.9656213396228257</v>
       </c>
       <c r="AC2" s="0">
-        <v>0.92595727247787962</v>
+        <v>0.92647699251782312</v>
       </c>
       <c r="AD2" s="0">
-        <v>0.99969155058838677</v>
+        <v>0.9998582321458569</v>
       </c>
       <c r="AE2" s="0">
-        <v>0.99402289444306691</v>
+        <v>0.99415901258958683</v>
       </c>
       <c r="AF2" s="0">
-        <v>0.89084867423245973</v>
+        <v>0.90576302655937457</v>
       </c>
       <c r="AG2" s="0">
-        <v>0.99087575652772353</v>
+        <v>0.9910719101256199</v>
       </c>
       <c r="AH2" s="0">
-        <v>0.99443053461312558</v>
+        <v>0.99457581578870336</v>
       </c>
       <c r="AI2" s="0">
-        <v>0.98432037083156088</v>
+        <v>0.98442918939531321</v>
       </c>
       <c r="AJ2" s="0">
-        <v>0.97601936707241066</v>
+        <v>0.97646953989857188</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
@@ -5347,52 +5347,52 @@
         <v>37</v>
       </c>
       <c r="B3" s="0">
-        <v>0.10648885198790194</v>
+        <v>0.10537965170389695</v>
       </c>
       <c r="C3" s="0">
-        <v>0.0040723012101617669</v>
+        <v>0.0040288097707927633</v>
       </c>
       <c r="D3" s="0">
-        <v>0.0095040030267806008</v>
+        <v>0.0094380505562253279</v>
       </c>
       <c r="E3" s="0">
-        <v>0.1083915720785881</v>
+        <v>0.10736226060685601</v>
       </c>
       <c r="F3" s="0">
-        <v>0.0085003142074023628</v>
+        <v>0.0084097175425268712</v>
       </c>
       <c r="G3" s="0">
-        <v>0.0044307763847099739</v>
+        <v>0.0043857522136883783</v>
       </c>
       <c r="H3" s="0">
-        <v>0.097914402769721673</v>
+        <v>0.09697558974902136</v>
       </c>
       <c r="I3" s="0">
-        <v>0.0049060810273028879</v>
+        <v>0.0048551523528208747</v>
       </c>
       <c r="J3" s="0">
-        <v>0.0091387070890891868</v>
+        <v>0.0090436947845803084</v>
       </c>
       <c r="K3" s="0">
-        <v>0.071759730777259598</v>
+        <v>0.071046639742007603</v>
       </c>
       <c r="L3" s="0">
-        <v>0.069434265444055565</v>
+        <v>0.068717255680316641</v>
       </c>
       <c r="M3" s="0">
-        <v>0.048377461242294161</v>
+        <v>0.047890885560054712</v>
       </c>
       <c r="N3" s="0">
-        <v>0.057089392364475591</v>
+        <v>0.05648075102183682</v>
       </c>
       <c r="O3" s="0">
-        <v>0.0083789275392315895</v>
+        <v>0.0082895438112914124</v>
       </c>
       <c r="P3" s="0">
-        <v>0.2388720144785518</v>
+        <v>0.23631620861679239</v>
       </c>
       <c r="Q3" s="0">
-        <v>0.0027666621789289949</v>
+        <v>0.0027373464546235071</v>
       </c>
       <c r="R3" s="0">
         <v>0</v>
@@ -5401,55 +5401,55 @@
         <v>0</v>
       </c>
       <c r="T3" s="0">
-        <v>0.0026406300831979955</v>
+        <v>0.0026153794310981673</v>
       </c>
       <c r="U3" s="0">
-        <v>0.010617652217454828</v>
+        <v>0.010506831788453542</v>
       </c>
       <c r="V3" s="0">
-        <v>0.006376092597168247</v>
+        <v>0.0063251247390434789</v>
       </c>
       <c r="W3" s="0">
-        <v>0.004476099003994741</v>
+        <v>0.0046445810172954412</v>
       </c>
       <c r="X3" s="0">
-        <v>0.0090912634686910482</v>
+        <v>0.0090050405513800586</v>
       </c>
       <c r="Y3" s="0">
-        <v>0.097755993953546033</v>
+        <v>0.096716879985893775</v>
       </c>
       <c r="Z3" s="0">
-        <v>0.068092639703748403</v>
+        <v>0.067418368064244991</v>
       </c>
       <c r="AA3" s="0">
-        <v>0.069322087922700337</v>
+        <v>0.068677021480574266</v>
       </c>
       <c r="AB3" s="0">
-        <v>0.033051216868963396</v>
+        <v>0.032714330327574447</v>
       </c>
       <c r="AC3" s="0">
-        <v>0.074024261038220879</v>
+        <v>0.073273305115649973</v>
       </c>
       <c r="AD3" s="0">
         <v>0</v>
       </c>
       <c r="AE3" s="0">
-        <v>0.0039277684996881839</v>
+        <v>0.0038862734770754026</v>
       </c>
       <c r="AF3" s="0">
-        <v>0.093687719970731206</v>
+        <v>0.094236973440625538</v>
       </c>
       <c r="AG3" s="0">
-        <v>0.0078120080033669175</v>
+        <v>0.0077299494343571352</v>
       </c>
       <c r="AH3" s="0">
-        <v>0.0018753282986914413</v>
+        <v>0.0018555333301528637</v>
       </c>
       <c r="AI3" s="0">
         <v>0</v>
       </c>
       <c r="AJ3" s="0">
-        <v>0.011119766720210072</v>
+        <v>0.011005859146942793</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
@@ -5457,61 +5457,61 @@
         <v>38</v>
       </c>
       <c r="B4" s="0">
-        <v>0</v>
+        <v>0.00085920010576578661</v>
       </c>
       <c r="C4" s="0">
-        <v>0.00079661688235210901</v>
+        <v>0.00082278465488138145</v>
       </c>
       <c r="D4" s="0">
-        <v>0.043764857622981657</v>
+        <v>0.043097106758626734</v>
       </c>
       <c r="E4" s="0">
         <v>0</v>
       </c>
       <c r="F4" s="0">
-        <v>0.0018551850916959905</v>
+        <v>0.0019057575243933687</v>
       </c>
       <c r="G4" s="0">
-        <v>0.0043964158005294863</v>
+        <v>0.0043521047132952986</v>
       </c>
       <c r="H4" s="0">
         <v>0</v>
       </c>
       <c r="I4" s="0">
-        <v>0.00039893024580591027</v>
+        <v>0.00044251494813721726</v>
       </c>
       <c r="J4" s="0">
-        <v>0.015561244407018879</v>
+        <v>0.015331452296253512</v>
       </c>
       <c r="K4" s="0">
         <v>0</v>
       </c>
       <c r="L4" s="0">
-        <v>0.0046847340871166787</v>
+        <v>0.0053220230066635963</v>
       </c>
       <c r="M4" s="0">
         <v>0</v>
       </c>
       <c r="N4" s="0">
-        <v>0.00071787752817273852</v>
+        <v>0.0013069687315010146</v>
       </c>
       <c r="O4" s="0">
-        <v>0.003213976987865018</v>
+        <v>0.003234366727722874</v>
       </c>
       <c r="P4" s="0">
-        <v>-0.045234060198447369</v>
+        <v>-0.041742670085451114</v>
       </c>
       <c r="Q4" s="0">
         <v>0</v>
       </c>
       <c r="R4" s="0">
-        <v>0.00030651424383336363</v>
+        <v>0.00026235144992769842</v>
       </c>
       <c r="S4" s="0">
         <v>0</v>
       </c>
       <c r="T4" s="0">
-        <v>0.0041048136045659612</v>
+        <v>0.004050044951939928</v>
       </c>
       <c r="U4" s="0">
         <v>0</v>
@@ -5520,31 +5520,31 @@
         <v>0</v>
       </c>
       <c r="W4" s="0">
-        <v>0.0032639165463509354</v>
+        <v>0.0034002301271040163</v>
       </c>
       <c r="X4" s="0">
         <v>0</v>
       </c>
       <c r="Y4" s="0">
-        <v>0.0009774895719105389</v>
+        <v>0.0019916218348393789</v>
       </c>
       <c r="Z4" s="0">
         <v>0</v>
       </c>
       <c r="AA4" s="0">
-        <v>0.0021545451826892538</v>
+        <v>0.0028465013995376161</v>
       </c>
       <c r="AB4" s="0">
-        <v>0.0013421823647126829</v>
+        <v>0.0016643300495999094</v>
       </c>
       <c r="AC4" s="0">
-        <v>0</v>
+        <v>0.00023855771514707781</v>
       </c>
       <c r="AD4" s="0">
-        <v>4.7577405624315246e-05</v>
+        <v>2.7627167693384927e-05</v>
       </c>
       <c r="AE4" s="0">
-        <v>0.0016614035170320698</v>
+        <v>0.0016678454864591454</v>
       </c>
       <c r="AF4" s="0">
         <v>0</v>
@@ -5556,10 +5556,10 @@
         <v>0</v>
       </c>
       <c r="AI4" s="0">
-        <v>0.012040242521909064</v>
+        <v>0.011782918888026709</v>
       </c>
       <c r="AJ4" s="0">
-        <v>0.00058493800191704412</v>
+        <v>0.00069051404141889992</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
@@ -5573,43 +5573,43 @@
         <v>0</v>
       </c>
       <c r="D5" s="0">
-        <v>0.0010931614486786047</v>
+        <v>0</v>
       </c>
       <c r="E5" s="0">
-        <v>3.7366477390101138e-05</v>
+        <v>0</v>
       </c>
       <c r="F5" s="0">
         <v>0</v>
       </c>
       <c r="G5" s="0">
-        <v>0.011291806567924351</v>
+        <v>0.01103178617824256</v>
       </c>
       <c r="H5" s="0">
-        <v>2.3066605897854904e-05</v>
+        <v>0</v>
       </c>
       <c r="I5" s="0">
         <v>0</v>
       </c>
       <c r="J5" s="0">
-        <v>0.00027019315065512293</v>
+        <v>0.00058875029717742478</v>
       </c>
       <c r="K5" s="0">
         <v>0</v>
       </c>
       <c r="L5" s="0">
-        <v>0.00076554865073297424</v>
+        <v>0.00084754027845014991</v>
       </c>
       <c r="M5" s="0">
-        <v>0.10813685809200982</v>
+        <v>0.10464605093483274</v>
       </c>
       <c r="N5" s="0">
         <v>0</v>
       </c>
       <c r="O5" s="0">
-        <v>0.00079759677186243565</v>
+        <v>0.00084055849573259781</v>
       </c>
       <c r="P5" s="0">
-        <v>0.0050410789410492603</v>
+        <v>0.0039606391838060764</v>
       </c>
       <c r="Q5" s="0">
         <v>0</v>
@@ -5618,22 +5618,22 @@
         <v>0</v>
       </c>
       <c r="S5" s="0">
-        <v>0.00027217718564501761</v>
+        <v>0</v>
       </c>
       <c r="T5" s="0">
-        <v>0.00052162276093001628</v>
+        <v>0</v>
       </c>
       <c r="U5" s="0">
-        <v>4.0936137312983313e-05</v>
+        <v>2.3217296318625041e-05</v>
       </c>
       <c r="V5" s="0">
         <v>0</v>
       </c>
       <c r="W5" s="0">
-        <v>0.00066873703035844653</v>
+        <v>0.00075137150772460002</v>
       </c>
       <c r="X5" s="0">
-        <v>9.3907145278461333e-05</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="0">
         <v>0</v>
@@ -5642,31 +5642,31 @@
         <v>0</v>
       </c>
       <c r="AA5" s="0">
-        <v>0.0087338614908911618</v>
+        <v>0.0085214673441352546</v>
       </c>
       <c r="AB5" s="0">
-        <v>0.00029621191341604094</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="0">
         <v>0</v>
       </c>
       <c r="AD5" s="0">
-        <v>4.3853127270399889e-05</v>
+        <v>4.3261465972303249e-05</v>
       </c>
       <c r="AE5" s="0">
-        <v>0.00018133735026301231</v>
+        <v>0.00021084948019903647</v>
       </c>
       <c r="AF5" s="0">
-        <v>0.010967329204202582</v>
+        <v>0</v>
       </c>
       <c r="AG5" s="0">
-        <v>0.00050558486585754907</v>
+        <v>0.00046593691511015944</v>
       </c>
       <c r="AH5" s="0">
-        <v>0.00015381516101290756</v>
+        <v>0.00012345525810068445</v>
       </c>
       <c r="AI5" s="0">
-        <v>0.0018418511824241067</v>
+        <v>0.0020357348190018151</v>
       </c>
       <c r="AJ5" s="0">
         <v>0</v>
@@ -5683,103 +5683,103 @@
         <v>0</v>
       </c>
       <c r="D6" s="0">
-        <v>0.0017516312102093562</v>
+        <v>0</v>
       </c>
       <c r="E6" s="0">
-        <v>8.0469540263875553e-05</v>
+        <v>7.7562135042965336e-05</v>
       </c>
       <c r="F6" s="0">
         <v>0</v>
       </c>
       <c r="G6" s="0">
-        <v>0.0007021175110660696</v>
+        <v>0.0010255426091446982</v>
       </c>
       <c r="H6" s="0">
-        <v>3.7900722755222648e-05</v>
+        <v>0</v>
       </c>
       <c r="I6" s="0">
         <v>0</v>
       </c>
       <c r="J6" s="0">
-        <v>0.00061513071516114675</v>
+        <v>0.00060304739188767888</v>
       </c>
       <c r="K6" s="0">
         <v>0</v>
       </c>
       <c r="L6" s="0">
-        <v>0.00029482041130424137</v>
+        <v>0.00030797208158858924</v>
       </c>
       <c r="M6" s="0">
-        <v>0.015095126027305884</v>
+        <v>0.017829843479501777</v>
       </c>
       <c r="N6" s="0">
-        <v>0.00039924517907509558</v>
+        <v>0.00038070984867863124</v>
       </c>
       <c r="O6" s="0">
-        <v>0.0011661056385869409</v>
+        <v>0.0011429093281059128</v>
       </c>
       <c r="P6" s="0">
-        <v>0.0059836774611622895</v>
+        <v>0.0058734236451490496</v>
       </c>
       <c r="Q6" s="0">
-        <v>6.6463906535260532e-05</v>
+        <v>0</v>
       </c>
       <c r="R6" s="0">
-        <v>6.1207980975005368e-05</v>
+        <v>0</v>
       </c>
       <c r="S6" s="0">
-        <v>0.00015135339411638025</v>
+        <v>0</v>
       </c>
       <c r="T6" s="0">
-        <v>0.00049337648675915752</v>
+        <v>0</v>
       </c>
       <c r="U6" s="0">
-        <v>1.5854025932517697e-05</v>
+        <v>1.6192848514282793e-05</v>
       </c>
       <c r="V6" s="0">
         <v>0</v>
       </c>
       <c r="W6" s="0">
-        <v>0.00015984522191945621</v>
+        <v>0.00018355129289014311</v>
       </c>
       <c r="X6" s="0">
-        <v>0.00038672842308173103</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="0">
         <v>0</v>
       </c>
       <c r="Z6" s="0">
-        <v>3.9806270146605814e-05</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="0">
-        <v>0.0008024998369494489</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="0">
-        <v>0.00010418219005030119</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="0">
         <v>0</v>
       </c>
       <c r="AD6" s="0">
-        <v>7.2546091641587513e-05</v>
+        <v>7.087922047712516e-05</v>
       </c>
       <c r="AE6" s="0">
-        <v>7.2878735693233644e-05</v>
+        <v>7.6018966679676332e-05</v>
       </c>
       <c r="AF6" s="0">
-        <v>0.0029622158741196575</v>
+        <v>0</v>
       </c>
       <c r="AG6" s="0">
-        <v>0.0001136706838171796</v>
+        <v>0.00012423670497968938</v>
       </c>
       <c r="AH6" s="0">
         <v>0</v>
       </c>
       <c r="AI6" s="0">
-        <v>0.00029143899723204942</v>
+        <v>0.00034049478733955987</v>
       </c>
       <c r="AJ6" s="0">
-        <v>0.0041491894336393</v>
+        <v>0.0039749465704036532</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
@@ -5796,40 +5796,40 @@
         <v>0</v>
       </c>
       <c r="E7" s="0">
-        <v>9.2285673936488398e-06</v>
+        <v>1.20723469574445e-05</v>
       </c>
       <c r="F7" s="0">
         <v>0</v>
       </c>
       <c r="G7" s="0">
-        <v>0.00042896084690501675</v>
+        <v>0</v>
       </c>
       <c r="H7" s="0">
         <v>0</v>
       </c>
       <c r="I7" s="0">
-        <v>1.7813746642282805e-05</v>
+        <v>1.5864721630745681e-05</v>
       </c>
       <c r="J7" s="0">
-        <v>6.8637847992754277e-05</v>
+        <v>9.0544412407530454e-05</v>
       </c>
       <c r="K7" s="0">
         <v>0</v>
       </c>
       <c r="L7" s="0">
-        <v>0.00045550474364295193</v>
+        <v>0.00044443835618308565</v>
       </c>
       <c r="M7" s="0">
-        <v>0.00090494349509153088</v>
+        <v>0.0015493144959857319</v>
       </c>
       <c r="N7" s="0">
-        <v>0.00014961871468378859</v>
+        <v>0.00015811819718094763</v>
       </c>
       <c r="O7" s="0">
-        <v>0.003232203871059912</v>
+        <v>0.0031113970371645797</v>
       </c>
       <c r="P7" s="0">
-        <v>0.12040703003971563</v>
+        <v>0.11435015515080384</v>
       </c>
       <c r="Q7" s="0">
         <v>0</v>
@@ -5838,46 +5838,46 @@
         <v>0</v>
       </c>
       <c r="S7" s="0">
-        <v>8.5306934021125752e-07</v>
+        <v>0</v>
       </c>
       <c r="T7" s="0">
-        <v>2.8516043916613601e-05</v>
+        <v>0</v>
       </c>
       <c r="U7" s="0">
-        <v>4.9936530641788761e-05</v>
+        <v>4.8007533043546317e-05</v>
       </c>
       <c r="V7" s="0">
-        <v>9.7215283546818603e-05</v>
+        <v>9.053987876202217e-05</v>
       </c>
       <c r="W7" s="0">
-        <v>0.00011225613359845525</v>
+        <v>0.00011893198331798023</v>
       </c>
       <c r="X7" s="0">
-        <v>0.00063462147826055901</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="0">
-        <v>1.9984585490013985e-05</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="0">
-        <v>6.4409408223540256e-06</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="0">
-        <v>0.0003091737252737492</v>
+        <v>0</v>
       </c>
       <c r="AB7" s="0">
-        <v>6.8537452341712763e-05</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="0">
-        <v>1.37130146688557e-05</v>
+        <v>1.1144651379813502e-05</v>
       </c>
       <c r="AD7" s="0">
-        <v>5.3376203448204764e-06</v>
+        <v>0</v>
       </c>
       <c r="AE7" s="0">
-        <v>6.0234351569389303e-05</v>
+        <v>0</v>
       </c>
       <c r="AF7" s="0">
-        <v>0.0014751691635734459</v>
+        <v>0</v>
       </c>
       <c r="AG7" s="0">
         <v>0</v>
@@ -5889,7 +5889,7 @@
         <v>0</v>
       </c>
       <c r="AJ7" s="0">
-        <v>0.0079600649758605896</v>
+        <v>0.0077168515970990493</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
@@ -5912,37 +5912,37 @@
         <v>0</v>
       </c>
       <c r="G8" s="0">
-        <v>1.584404239625747e-05</v>
+        <v>0</v>
       </c>
       <c r="H8" s="0">
         <v>0</v>
       </c>
       <c r="I8" s="0">
-        <v>4.1810703197013747e-06</v>
+        <v>0</v>
       </c>
       <c r="J8" s="0">
-        <v>6.7930922733727529e-05</v>
+        <v>0</v>
       </c>
       <c r="K8" s="0">
         <v>0</v>
       </c>
       <c r="L8" s="0">
-        <v>6.219089612799379e-05</v>
+        <v>0</v>
       </c>
       <c r="M8" s="0">
-        <v>0.00011903890296466489</v>
+        <v>0.00017542784408366717</v>
       </c>
       <c r="N8" s="0">
-        <v>1.7001818005441316e-05</v>
+        <v>2.3962565187116887e-05</v>
       </c>
       <c r="O8" s="0">
-        <v>0.0026282510657503894</v>
+        <v>0.0026292088991244512</v>
       </c>
       <c r="P8" s="0">
-        <v>-0.032236489955994291</v>
+        <v>-0.024110440966529097</v>
       </c>
       <c r="Q8" s="0">
-        <v>2.3802337872733091e-06</v>
+        <v>0</v>
       </c>
       <c r="R8" s="0">
         <v>0</v>
@@ -5954,25 +5954,25 @@
         <v>0</v>
       </c>
       <c r="U8" s="0">
-        <v>2.6737252111805013e-05</v>
+        <v>2.7622838376439866e-05</v>
       </c>
       <c r="V8" s="0">
-        <v>0.00012767297677403661</v>
+        <v>0.0001249131417522438</v>
       </c>
       <c r="W8" s="0">
-        <v>4.0167349720802803e-05</v>
+        <v>4.5658329325754061e-05</v>
       </c>
       <c r="X8" s="0">
         <v>0</v>
       </c>
       <c r="Y8" s="0">
-        <v>5.9938649055458564e-06</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="0">
-        <v>2.0470970795926481e-05</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="0">
-        <v>3.7098972999138222e-06</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="0">
         <v>0</v>
@@ -5981,22 +5981,22 @@
         <v>0</v>
       </c>
       <c r="AD8" s="0">
-        <v>4.2696600918828721e-05</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="0">
-        <v>9.5939344270262303e-06</v>
+        <v>0</v>
       </c>
       <c r="AF8" s="0">
         <v>0</v>
       </c>
       <c r="AG8" s="0">
-        <v>0.00011226739997034734</v>
+        <v>8.5737895481421039e-05</v>
       </c>
       <c r="AH8" s="0">
-        <v>0.0001920000028858209</v>
+        <v>0.0001782135561388427</v>
       </c>
       <c r="AI8" s="0">
-        <v>0.00018817769622330162</v>
+        <v>0.00012075267816703545</v>
       </c>
       <c r="AJ8" s="0">
         <v>0</v>
@@ -6007,76 +6007,76 @@
         <v>43</v>
       </c>
       <c r="B9" s="0">
-        <v>5.6460520789047058e-06</v>
+        <v>0</v>
       </c>
       <c r="C9" s="0">
-        <v>2.9556903025828236e-06</v>
+        <v>0</v>
       </c>
       <c r="D9" s="0">
-        <v>7.3819106308147138e-06</v>
+        <v>0</v>
       </c>
       <c r="E9" s="0">
-        <v>1.5178630148095746e-05</v>
+        <v>0</v>
       </c>
       <c r="F9" s="0">
-        <v>1.9359070528620861e-06</v>
+        <v>0</v>
       </c>
       <c r="G9" s="0">
-        <v>6.1339908403323243e-05</v>
+        <v>0</v>
       </c>
       <c r="H9" s="0">
-        <v>1.2086675904030025e-05</v>
+        <v>0</v>
       </c>
       <c r="I9" s="0">
-        <v>0.0001255970101578947</v>
+        <v>0</v>
       </c>
       <c r="J9" s="0">
-        <v>0.0002113312725190978</v>
+        <v>0</v>
       </c>
       <c r="K9" s="0">
-        <v>2.0446502565440125e-06</v>
+        <v>0</v>
       </c>
       <c r="L9" s="0">
-        <v>0.00027577683156412082</v>
+        <v>0</v>
       </c>
       <c r="M9" s="0">
-        <v>4.4127458598742422e-05</v>
+        <v>4.9971117022791698e-05</v>
       </c>
       <c r="N9" s="0">
-        <v>0.00020283267663343202</v>
+        <v>0.0001894031411418202</v>
       </c>
       <c r="O9" s="0">
-        <v>0.00028569115364930489</v>
+        <v>0.00042845600079127039</v>
       </c>
       <c r="P9" s="0">
-        <v>-0.0039443325429986548</v>
+        <v>-0.0054023464231868993</v>
       </c>
       <c r="Q9" s="0">
         <v>0</v>
       </c>
       <c r="R9" s="0">
-        <v>4.2973822239603122e-05</v>
+        <v>0</v>
       </c>
       <c r="S9" s="0">
-        <v>4.9896093779108527e-06</v>
+        <v>0</v>
       </c>
       <c r="T9" s="0">
-        <v>1.1862751282931521e-05</v>
+        <v>0</v>
       </c>
       <c r="U9" s="0">
-        <v>1.9497192711110263e-05</v>
+        <v>1.9779035212035885e-05</v>
       </c>
       <c r="V9" s="0">
-        <v>8.8321290880701057e-06</v>
+        <v>1.6076750671408087e-05</v>
       </c>
       <c r="W9" s="0">
-        <v>3.0053366554445737e-05</v>
+        <v>3.1966701977480259e-05</v>
       </c>
       <c r="X9" s="0">
         <v>0</v>
       </c>
       <c r="Y9" s="0">
-        <v>1.1279473641441528e-05</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="0">
         <v>0</v>
@@ -6085,28 +6085,28 @@
         <v>0</v>
       </c>
       <c r="AB9" s="0">
-        <v>6.9433511071512132e-06</v>
+        <v>0</v>
       </c>
       <c r="AC9" s="0">
-        <v>1.5912575648000458e-06</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="0">
-        <v>9.263611208758616e-05</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="0">
-        <v>6.2580162347774696e-05</v>
+        <v>0</v>
       </c>
       <c r="AF9" s="0">
-        <v>3.8893772599296519e-06</v>
+        <v>0</v>
       </c>
       <c r="AG9" s="0">
         <v>0</v>
       </c>
       <c r="AH9" s="0">
-        <v>2.2968381952155059e-05</v>
+        <v>3.2806539088185046e-05</v>
       </c>
       <c r="AI9" s="0">
-        <v>4.58545871497606e-05</v>
+        <v>5.2069014446384599e-05</v>
       </c>
       <c r="AJ9" s="0">
         <v>0</v>
@@ -6117,16 +6117,16 @@
         <v>44</v>
       </c>
       <c r="B10" s="0">
-        <v>7.2992949115162666e-07</v>
+        <v>0</v>
       </c>
       <c r="C10" s="0">
         <v>0</v>
       </c>
       <c r="D10" s="0">
-        <v>2.002227644186426e-06</v>
+        <v>0</v>
       </c>
       <c r="E10" s="0">
-        <v>2.6488125007682601e-06</v>
+        <v>0</v>
       </c>
       <c r="F10" s="0">
         <v>0</v>
@@ -6135,22 +6135,22 @@
         <v>0</v>
       </c>
       <c r="H10" s="0">
-        <v>1.8853254304120829e-06</v>
+        <v>0</v>
       </c>
       <c r="I10" s="0">
-        <v>0.00017818941886386347</v>
+        <v>0</v>
       </c>
       <c r="J10" s="0">
-        <v>2.2077447631507763e-05</v>
+        <v>0</v>
       </c>
       <c r="K10" s="0">
-        <v>5.6984610312896816e-07</v>
+        <v>0</v>
       </c>
       <c r="L10" s="0">
-        <v>1.4011512813008643e-05</v>
+        <v>0</v>
       </c>
       <c r="M10" s="0">
-        <v>4.1660218156852952e-05</v>
+        <v>4.1629258776601951e-05</v>
       </c>
       <c r="N10" s="0">
         <v>0</v>
@@ -6159,46 +6159,46 @@
         <v>0</v>
       </c>
       <c r="P10" s="0">
-        <v>0.0022050612677944215</v>
+        <v>0.0016814616308938113</v>
       </c>
       <c r="Q10" s="0">
-        <v>5.171346175404893e-06</v>
+        <v>0</v>
       </c>
       <c r="R10" s="0">
-        <v>9.9931372053730996e-06</v>
+        <v>0</v>
       </c>
       <c r="S10" s="0">
-        <v>1.5211549575969961e-06</v>
+        <v>0</v>
       </c>
       <c r="T10" s="0">
-        <v>5.5055428113739613e-06</v>
+        <v>0</v>
       </c>
       <c r="U10" s="0">
         <v>0</v>
       </c>
       <c r="V10" s="0">
-        <v>0.00010574805985327543</v>
+        <v>9.8201026828642597e-05</v>
       </c>
       <c r="W10" s="0">
-        <v>0.00022002967617521923</v>
+        <v>0.00021403991955625811</v>
       </c>
       <c r="X10" s="0">
-        <v>1.4859895039602349e-05</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="0">
         <v>0</v>
       </c>
       <c r="Z10" s="0">
-        <v>7.3562865579426812e-06</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="0">
-        <v>9.9797639209253125e-06</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="0">
-        <v>4.0834686503475566e-06</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="0">
-        <v>2.9702832778703119e-06</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="0">
         <v>0</v>
@@ -6207,19 +6207,19 @@
         <v>0</v>
       </c>
       <c r="AF10" s="0">
-        <v>5.4571776421922018e-05</v>
+        <v>0</v>
       </c>
       <c r="AG10" s="0">
-        <v>0.00024732841569319986</v>
+        <v>0.0002255911159295017</v>
       </c>
       <c r="AH10" s="0">
         <v>0</v>
       </c>
       <c r="AI10" s="0">
-        <v>2.4543241548702723e-05</v>
+        <v>2.6087009125807412e-05</v>
       </c>
       <c r="AJ10" s="0">
-        <v>0.00016577713112052268</v>
+        <v>0.00013147855399070808</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
@@ -6266,13 +6266,13 @@
         <v>0</v>
       </c>
       <c r="O11" s="0">
-        <v>4.9223031635656283e-06</v>
+        <v>0</v>
       </c>
       <c r="P11" s="0">
-        <v>2.4439615888103901e-05</v>
+        <v>0.00018167696331588686</v>
       </c>
       <c r="Q11" s="0">
-        <v>1.3935683740249601e-06</v>
+        <v>0</v>
       </c>
       <c r="R11" s="0">
         <v>0</v>
@@ -6284,25 +6284,25 @@
         <v>0</v>
       </c>
       <c r="U11" s="0">
-        <v>2.6859443528551532e-08</v>
+        <v>0</v>
       </c>
       <c r="V11" s="0">
         <v>0</v>
       </c>
       <c r="W11" s="0">
-        <v>0.00016816639398401585</v>
+        <v>0</v>
       </c>
       <c r="X11" s="0">
         <v>0</v>
       </c>
       <c r="Y11" s="0">
-        <v>1.0197734019738657e-06</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="0">
-        <v>2.9791106535741545e-06</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="0">
-        <v>4.1484700298855388e-06</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="0">
         <v>0</v>
@@ -6323,13 +6323,13 @@
         <v>0</v>
       </c>
       <c r="AH11" s="0">
-        <v>5.0085060178719735e-06</v>
+        <v>1.1939670581655611e-06</v>
       </c>
       <c r="AI11" s="0">
         <v>0</v>
       </c>
       <c r="AJ11" s="0">
-        <v>0</v>
+        <v>1.0529003396597042e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
@@ -6340,19 +6340,19 @@
         <v>0</v>
       </c>
       <c r="C12" s="0">
-        <v>1.3658047534942004e-08</v>
+        <v>0</v>
       </c>
       <c r="D12" s="0">
         <v>0</v>
       </c>
       <c r="E12" s="0">
-        <v>3.5600859222260837e-08</v>
+        <v>0</v>
       </c>
       <c r="F12" s="0">
-        <v>1.2245304539448757e-08</v>
+        <v>0</v>
       </c>
       <c r="G12" s="0">
-        <v>4.4819679411993237e-07</v>
+        <v>0</v>
       </c>
       <c r="H12" s="0">
         <v>0</v>
@@ -6361,25 +6361,25 @@
         <v>0</v>
       </c>
       <c r="J12" s="0">
-        <v>4.3703113059356592e-07</v>
+        <v>0</v>
       </c>
       <c r="K12" s="0">
         <v>0</v>
       </c>
       <c r="L12" s="0">
-        <v>8.0159574653873996e-07</v>
+        <v>0</v>
       </c>
       <c r="M12" s="0">
-        <v>6.3809625276261345e-07</v>
+        <v>0</v>
       </c>
       <c r="N12" s="0">
-        <v>3.6664847845315278e-06</v>
+        <v>2.4932396960406954e-06</v>
       </c>
       <c r="O12" s="0">
-        <v>5.5579450699008167e-06</v>
+        <v>4.7686419641022104e-06</v>
       </c>
       <c r="P12" s="0">
-        <v>-0.00010628476401837095</v>
+        <v>-8.5393561441663181e-05</v>
       </c>
       <c r="Q12" s="0">
         <v>0</v>
@@ -6394,19 +6394,19 @@
         <v>0</v>
       </c>
       <c r="U12" s="0">
-        <v>5.7407992453449849e-07</v>
+        <v>0</v>
       </c>
       <c r="V12" s="0">
-        <v>0.0024424377359715003</v>
+        <v>0</v>
       </c>
       <c r="W12" s="0">
-        <v>0.0041584078384166228</v>
+        <v>0</v>
       </c>
       <c r="X12" s="0">
         <v>0</v>
       </c>
       <c r="Y12" s="0">
-        <v>8.09353498500883e-07</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="0">
         <v>0</v>
@@ -6418,13 +6418,13 @@
         <v>0</v>
       </c>
       <c r="AC12" s="0">
-        <v>4.8372845291371829e-08</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="0">
-        <v>3.8024537256211964e-06</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="0">
-        <v>1.3090059123402207e-06</v>
+        <v>0</v>
       </c>
       <c r="AF12" s="0">
         <v>0</v>
@@ -6433,10 +6433,10 @@
         <v>0</v>
       </c>
       <c r="AH12" s="0">
-        <v>0.0026720646731540204</v>
+        <v>0.0024001604122786549</v>
       </c>
       <c r="AI12" s="0">
-        <v>0.0009980650066323401</v>
+        <v>0.00089526199688677057</v>
       </c>
       <c r="AJ12" s="0">
         <v>0</v>
@@ -6447,73 +6447,73 @@
         <v>47</v>
       </c>
       <c r="B13" s="0">
-        <v>1.8556011732157103e-08</v>
+        <v>0</v>
       </c>
       <c r="C13" s="0">
-        <v>6.9897706649259023e-09</v>
+        <v>0</v>
       </c>
       <c r="D13" s="0">
-        <v>1.4132221161527935e-08</v>
+        <v>0</v>
       </c>
       <c r="E13" s="0">
-        <v>1.1735876217366842e-07</v>
+        <v>0</v>
       </c>
       <c r="F13" s="0">
-        <v>4.963863476812551e-09</v>
+        <v>0</v>
       </c>
       <c r="G13" s="0">
-        <v>4.703660215123427e-09</v>
+        <v>0</v>
       </c>
       <c r="H13" s="0">
-        <v>4.144148188106131e-08</v>
+        <v>0</v>
       </c>
       <c r="I13" s="0">
-        <v>3.6500167287129001e-06</v>
+        <v>0</v>
       </c>
       <c r="J13" s="0">
-        <v>4.3192654774705489e-07</v>
+        <v>0</v>
       </c>
       <c r="K13" s="0">
-        <v>8.9344999389838755e-09</v>
+        <v>0</v>
       </c>
       <c r="L13" s="0">
-        <v>4.6912759965924722e-07</v>
+        <v>0</v>
       </c>
       <c r="M13" s="0">
-        <v>1.5684273983132173e-06</v>
+        <v>1.3376494959005055e-06</v>
       </c>
       <c r="N13" s="0">
-        <v>7.3864393307844227e-08</v>
+        <v>3.7825629992899198e-07</v>
       </c>
       <c r="O13" s="0">
         <v>0</v>
       </c>
       <c r="P13" s="0">
-        <v>6.0222808722403303e-06</v>
+        <v>-4.4617620386685393e-06</v>
       </c>
       <c r="Q13" s="0">
         <v>0</v>
       </c>
       <c r="R13" s="0">
-        <v>2.8492122053337227e-07</v>
+        <v>0</v>
       </c>
       <c r="S13" s="0">
-        <v>2.0734156066037129e-08</v>
+        <v>0</v>
       </c>
       <c r="T13" s="0">
-        <v>6.1075420339690451e-08</v>
+        <v>0</v>
       </c>
       <c r="U13" s="0">
         <v>0</v>
       </c>
       <c r="V13" s="0">
-        <v>0.00020692097806885275</v>
+        <v>0</v>
       </c>
       <c r="W13" s="0">
-        <v>0.042242009396982569</v>
+        <v>0</v>
       </c>
       <c r="X13" s="0">
-        <v>7.2681865336935454e-08</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="0">
         <v>0</v>
@@ -6525,10 +6525,10 @@
         <v>0</v>
       </c>
       <c r="AB13" s="0">
-        <v>4.3625681385836951e-08</v>
+        <v>0</v>
       </c>
       <c r="AC13" s="0">
-        <v>1.4355554263456389e-07</v>
+        <v>0</v>
       </c>
       <c r="AD13" s="0">
         <v>0</v>
@@ -6537,19 +6537,19 @@
         <v>0</v>
       </c>
       <c r="AF13" s="0">
-        <v>3.5000210714870299e-07</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="0">
-        <v>3.9295066725819371e-05</v>
+        <v>3.4047128977057849e-05</v>
       </c>
       <c r="AH13" s="0">
-        <v>0.00064828036316032071</v>
+        <v>0.00083282114847901573</v>
       </c>
       <c r="AI13" s="0">
-        <v>0.00024945593531966031</v>
+        <v>0.00031749141169294676</v>
       </c>
       <c r="AJ13" s="0">
-        <v>5.9863084763709928e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
@@ -6563,7 +6563,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="0">
-        <v>9.3697133503289591e-10</v>
+        <v>0</v>
       </c>
       <c r="E14" s="0">
         <v>0</v>
@@ -6584,13 +6584,13 @@
         <v>0</v>
       </c>
       <c r="K14" s="0">
-        <v>2.7156847982198585e-10</v>
+        <v>0</v>
       </c>
       <c r="L14" s="0">
         <v>0</v>
       </c>
       <c r="M14" s="0">
-        <v>0</v>
+        <v>2.1034357733283771e-08</v>
       </c>
       <c r="N14" s="0">
         <v>0</v>
@@ -6599,22 +6599,22 @@
         <v>0</v>
       </c>
       <c r="P14" s="0">
-        <v>4.2239720803714554e-06</v>
+        <v>3.7541085627019723e-06</v>
       </c>
       <c r="Q14" s="0">
-        <v>3.8669579622730771e-08</v>
+        <v>0</v>
       </c>
       <c r="R14" s="0">
         <v>0</v>
       </c>
       <c r="S14" s="0">
-        <v>7.2023888461247486e-10</v>
+        <v>0</v>
       </c>
       <c r="T14" s="0">
-        <v>4.8058624013340282e-09</v>
+        <v>0</v>
       </c>
       <c r="U14" s="0">
-        <v>0.00013300677722441563</v>
+        <v>0</v>
       </c>
       <c r="V14" s="0">
         <v>0</v>
@@ -6623,19 +6623,19 @@
         <v>0</v>
       </c>
       <c r="X14" s="0">
-        <v>2.4365696078376991e-08</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="0">
         <v>0</v>
       </c>
       <c r="Z14" s="0">
-        <v>6.4464128046483172e-08</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="0">
-        <v>4.8210538620339705e-08</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="0">
-        <v>3.8534885553527826e-09</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="0">
         <v>0</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="AF14" s="0">
-        <v>8.0399124449427917e-08</v>
+        <v>0</v>
       </c>
       <c r="AG14" s="0">
-        <v>0.00029408903684541906</v>
+        <v>0.00026259067954511657</v>
       </c>
       <c r="AH14" s="0">
         <v>0</v>
@@ -6659,7 +6659,7 @@
         <v>0</v>
       </c>
       <c r="AJ14" s="0">
-        <v>2.9803399408935961e-07</v>
+        <v>2.8118817627501529e-07</v>
       </c>
     </row>
   </sheetData>
@@ -6689,7 +6689,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="0">
-        <v>0.035496283995967312</v>
+        <v>0.035699350638476173</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
@@ -6697,7 +6697,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="0">
-        <v>0.0028327674874329923</v>
+        <v>0.002837189540277763</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
@@ -6705,7 +6705,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="0">
-        <v>0.048516859136371958</v>
+        <v>0.0478161320367394</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
@@ -6713,7 +6713,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="0">
-        <v>0.021774338501756429</v>
+        <v>0.02154657417636302</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
@@ -6721,7 +6721,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="0">
-        <v>0.0030526710976985861</v>
+        <v>0.0030553081478284019</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
@@ -6729,7 +6729,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="0">
-        <v>0.012476874433451572</v>
+        <v>0.01257187265289636</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
@@ -6737,7 +6737,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="0">
-        <v>0.048957201384860836</v>
+        <v>0.04848779487451068</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
@@ -6745,7 +6745,7 @@
         <v>14</v>
       </c>
       <c r="B9" s="0">
-        <v>0.0011586020504252244</v>
+        <v>0.0011639011714498076</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
@@ -6753,7 +6753,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="0">
-        <v>0.0087750974911401346</v>
+        <v>0.008867552379641595</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
@@ -6761,7 +6761,7 @@
         <v>16</v>
       </c>
       <c r="B11" s="0">
-        <v>0.01435194615545192</v>
+        <v>0.014209327948401521</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
@@ -6769,7 +6769,7 @@
         <v>17</v>
       </c>
       <c r="B12" s="0">
-        <v>0.016911436986783913</v>
+        <v>0.017071600527252814</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
@@ -6795,7 +6795,7 @@
         <v>18</v>
       </c>
       <c r="B16" s="0">
-        <v>0.00092222072630966493</v>
+        <v>0.00091244881820783574</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
@@ -6803,7 +6803,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="0">
-        <v>0.00030651424383336363</v>
+        <v>0.00026235144992769842</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
@@ -6819,7 +6819,7 @@
         <v>21</v>
       </c>
       <c r="B19" s="0">
-        <v>0.0054251286461649588</v>
+        <v>0.0053577346674890114</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
@@ -6827,7 +6827,7 @@
         <v>22</v>
       </c>
       <c r="B20" s="0">
-        <v>0.0012611894425525727</v>
+        <v>0.0012428314459363521</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
@@ -6835,7 +6835,7 @@
         <v>23</v>
       </c>
       <c r="B21" s="0">
-        <v>0.0010670020322486567</v>
+        <v>0.0010531810565870064</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
@@ -6843,7 +6843,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="0">
-        <v>0.0020528024771312181</v>
+        <v>0.0021547571411343375</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
@@ -6851,7 +6851,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="0">
-        <v>0.0045456317343455241</v>
+        <v>0.0045025202756900293</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
@@ -6859,7 +6859,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="0">
-        <v>0.024927743274341777</v>
+        <v>0.025175030913893132</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
@@ -6867,7 +6867,7 @@
         <v>27</v>
       </c>
       <c r="B25" s="0">
-        <v>0.022697546567916133</v>
+        <v>0.022472789354748331</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
@@ -6875,7 +6875,7 @@
         <v>28</v>
       </c>
       <c r="B26" s="0">
-        <v>0.033277587586917443</v>
+        <v>0.033311475437351752</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
@@ -6883,7 +6883,7 @@
         <v>29</v>
       </c>
       <c r="B27" s="0">
-        <v>0.017867790799194382</v>
+        <v>0.018021495213387133</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
@@ -6891,7 +6891,7 @@
         <v>30</v>
       </c>
       <c r="B28" s="0">
-        <v>0.014818565222313031</v>
+        <v>0.014761228760568641</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
@@ -6899,7 +6899,7 @@
         <v>31</v>
       </c>
       <c r="B29" s="0">
-        <v>0.00012922463990654506</v>
+        <v>0.00011713890380304506</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
@@ -6907,7 +6907,7 @@
         <v>32</v>
       </c>
       <c r="B30" s="0">
-        <v>0.002021525631828574</v>
+        <v>0.002039647189327377</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
@@ -6915,7 +6915,7 @@
         <v>33</v>
       </c>
       <c r="B31" s="0">
-        <v>0.046843859985365603</v>
+        <v>0.047118486720312769</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">

</xml_diff>